<commit_message>
Últimas alterações antes de uma mudança dŕastica, utilizando como save.
</commit_message>
<xml_diff>
--- a/Vendas_Do_Dia.xlsx
+++ b/Vendas_Do_Dia.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="35">
   <si>
     <t>Código</t>
   </si>
@@ -28,91 +28,97 @@
     <t>Código_Vendedor</t>
   </si>
   <si>
-    <t>05/03/2026</t>
+    <t>18/03/2026</t>
+  </si>
+  <si>
+    <t>Marcos Vinicius</t>
+  </si>
+  <si>
+    <t>Jerques</t>
+  </si>
+  <si>
+    <t>Sebastião</t>
+  </si>
+  <si>
+    <t>Michel</t>
+  </si>
+  <si>
+    <t>Caíque Mansur</t>
+  </si>
+  <si>
+    <t>Kenia</t>
   </si>
   <si>
     <t>Filipe Assis</t>
   </si>
   <si>
-    <t>Michel</t>
-  </si>
-  <si>
-    <t>Juliana</t>
-  </si>
-  <si>
     <t>Ian</t>
   </si>
   <si>
-    <t>Joseph</t>
+    <t>Suene</t>
+  </si>
+  <si>
+    <t>Camilo</t>
+  </si>
+  <si>
+    <t>Álvaro</t>
+  </si>
+  <si>
+    <t>Victor Prazeres</t>
+  </si>
+  <si>
+    <t>Davidson</t>
+  </si>
+  <si>
+    <t>Lorrane</t>
+  </si>
+  <si>
+    <t>Narjara</t>
+  </si>
+  <si>
+    <t>Monique</t>
+  </si>
+  <si>
+    <t>Guilherme</t>
+  </si>
+  <si>
+    <t>Ana Luiza</t>
   </si>
   <si>
     <t>Luis Felipe</t>
   </si>
   <si>
-    <t>Suene</t>
-  </si>
-  <si>
-    <t>Álvaro</t>
+    <t>Victor Pereira</t>
+  </si>
+  <si>
+    <t>Wellinton</t>
+  </si>
+  <si>
+    <t>Aurélio</t>
+  </si>
+  <si>
+    <t>Paulo</t>
+  </si>
+  <si>
+    <t>Robson</t>
   </si>
   <si>
     <t>Maycon</t>
   </si>
   <si>
-    <t>Victor Pereira</t>
-  </si>
-  <si>
-    <t>Samuel</t>
-  </si>
-  <si>
-    <t>Wellinton</t>
-  </si>
-  <si>
-    <t>Guilherme</t>
-  </si>
-  <si>
-    <t>Ana Luiza</t>
-  </si>
-  <si>
-    <t>Paulo</t>
-  </si>
-  <si>
-    <t>Aurélio</t>
-  </si>
-  <si>
-    <t>Cadu</t>
-  </si>
-  <si>
-    <t>Edson</t>
-  </si>
-  <si>
-    <t>Marcão</t>
-  </si>
-  <si>
-    <t>Janaína</t>
-  </si>
-  <si>
-    <t>Davidson</t>
-  </si>
-  <si>
-    <t>Kenia</t>
-  </si>
-  <si>
-    <t>Monique</t>
+    <t>Alisson</t>
+  </si>
+  <si>
+    <t>Bruno</t>
+  </si>
+  <si>
+    <t>Caio Edson</t>
+  </si>
+  <si>
+    <t>Daniele</t>
   </si>
   <si>
     <t>Alexandre</t>
-  </si>
-  <si>
-    <t>Marcos Vinicius</t>
-  </si>
-  <si>
-    <t>Camilo</t>
-  </si>
-  <si>
-    <t>Robson</t>
-  </si>
-  <si>
-    <t>Daniele</t>
   </si>
 </sst>
 </file>
@@ -471,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D168"/>
+  <dimension ref="A1:D178"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -494,7 +500,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1">
-        <v>6882831</v>
+        <v>6560577</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -503,12 +509,12 @@
         <v>5</v>
       </c>
       <c r="D2" s="1">
-        <v>502</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1">
-        <v>6416430</v>
+        <v>6938561</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -517,12 +523,12 @@
         <v>5</v>
       </c>
       <c r="D3" s="1">
-        <v>502</v>
+        <v>404</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1">
-        <v>7553536</v>
+        <v>6023751</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -531,12 +537,12 @@
         <v>5</v>
       </c>
       <c r="D4" s="1">
-        <v>502</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1">
-        <v>5351345</v>
+        <v>7535398</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -545,208 +551,208 @@
         <v>5</v>
       </c>
       <c r="D5" s="1">
-        <v>502</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1">
-        <v>5362565</v>
+        <v>5976217</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="1">
-        <v>502</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1">
-        <v>5416026</v>
+        <v>6933444</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1">
-        <v>5346706</v>
+        <v>3664967</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1">
-        <v>5859351</v>
+        <v>5398731</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1">
-        <v>5429545</v>
+        <v>7576963</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1">
-        <v>6392364</v>
+        <v>3290202</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D11" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1">
-        <v>645063</v>
+        <v>3324270</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D12" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1">
-        <v>5362579</v>
+        <v>6962447</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1">
-        <v>5362567</v>
+        <v>6929705</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D14" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1">
-        <v>6976608</v>
+        <v>7409406</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" s="1">
-        <v>502</v>
+        <v>401</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1">
-        <v>718714</v>
+        <v>3452176</v>
       </c>
       <c r="B16" t="s">
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D16" s="1">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1">
-        <v>7103745</v>
+        <v>3331471</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D17" s="1">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="1">
-        <v>653435</v>
+        <v>6954098</v>
       </c>
       <c r="B18" t="s">
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D18" s="1">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1">
-        <v>7303410</v>
+        <v>7332052</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" s="1">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1">
-        <v>6751368</v>
+        <v>7568265</v>
       </c>
       <c r="B20" t="s">
         <v>4</v>
@@ -755,82 +761,82 @@
         <v>7</v>
       </c>
       <c r="D20" s="1">
-        <v>153</v>
+        <v>401</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1">
-        <v>6584120</v>
+        <v>652507</v>
       </c>
       <c r="B21" t="s">
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D21" s="1">
-        <v>153</v>
+        <v>402</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1">
-        <v>7330434</v>
+        <v>2903112</v>
       </c>
       <c r="B22" t="s">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D22" s="1">
-        <v>153</v>
+        <v>402</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1">
-        <v>6165494</v>
+        <v>3587027</v>
       </c>
       <c r="B23" t="s">
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D23" s="1">
-        <v>153</v>
+        <v>402</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="1">
-        <v>7483627</v>
+        <v>6562716</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D24" s="1">
-        <v>153</v>
+        <v>402</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1">
-        <v>629604</v>
+        <v>3215539</v>
       </c>
       <c r="B25" t="s">
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D25" s="1">
-        <v>153</v>
+        <v>402</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="1">
-        <v>7087000</v>
+        <v>6260739</v>
       </c>
       <c r="B26" t="s">
         <v>4</v>
@@ -839,12 +845,12 @@
         <v>8</v>
       </c>
       <c r="D26" s="1">
-        <v>301</v>
+        <v>402</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="1">
-        <v>7483350</v>
+        <v>7523946</v>
       </c>
       <c r="B27" t="s">
         <v>4</v>
@@ -853,12 +859,12 @@
         <v>8</v>
       </c>
       <c r="D27" s="1">
-        <v>301</v>
+        <v>402</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="1">
-        <v>5485593</v>
+        <v>5729276</v>
       </c>
       <c r="B28" t="s">
         <v>4</v>
@@ -867,12 +873,12 @@
         <v>8</v>
       </c>
       <c r="D28" s="1">
-        <v>301</v>
+        <v>402</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="1">
-        <v>7408988</v>
+        <v>7288549</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
@@ -881,26 +887,26 @@
         <v>9</v>
       </c>
       <c r="D29" s="1">
-        <v>602</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="1">
-        <v>620045</v>
+        <v>6459199</v>
       </c>
       <c r="B30" t="s">
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D30" s="1">
-        <v>602</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1">
-        <v>6199900</v>
+        <v>4993036</v>
       </c>
       <c r="B31" t="s">
         <v>4</v>
@@ -909,12 +915,12 @@
         <v>10</v>
       </c>
       <c r="D31" s="1">
-        <v>505</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1">
-        <v>6147465</v>
+        <v>6121904</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
@@ -923,12 +929,12 @@
         <v>10</v>
       </c>
       <c r="D32" s="1">
-        <v>505</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1">
-        <v>5173892</v>
+        <v>6703859</v>
       </c>
       <c r="B33" t="s">
         <v>4</v>
@@ -937,12 +943,12 @@
         <v>10</v>
       </c>
       <c r="D33" s="1">
-        <v>505</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1">
-        <v>6345583</v>
+        <v>6802435</v>
       </c>
       <c r="B34" t="s">
         <v>4</v>
@@ -951,12 +957,12 @@
         <v>10</v>
       </c>
       <c r="D34" s="1">
-        <v>505</v>
+        <v>134</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1">
-        <v>5178184</v>
+        <v>6752243</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
@@ -965,110 +971,110 @@
         <v>10</v>
       </c>
       <c r="D35" s="1">
-        <v>505</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1">
-        <v>7056964</v>
+        <v>7396713</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D36" s="1">
-        <v>505</v>
+        <v>308</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="1">
-        <v>7372090</v>
+        <v>2850271</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D37" s="1">
-        <v>505</v>
+        <v>308</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1">
-        <v>5171245</v>
+        <v>7066398</v>
       </c>
       <c r="B38" t="s">
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D38" s="1">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1">
-        <v>5181870</v>
+        <v>6163577</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D39" s="1">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1">
-        <v>619674</v>
+        <v>7288831</v>
       </c>
       <c r="B40" t="s">
         <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D40" s="1">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1">
-        <v>7079157</v>
+        <v>7553536</v>
       </c>
       <c r="B41" t="s">
         <v>4</v>
       </c>
       <c r="C41" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D41" s="1">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="1">
-        <v>5692418</v>
+        <v>7236527</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
       </c>
       <c r="C42" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D42" s="1">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1">
-        <v>6968147</v>
+        <v>7522960</v>
       </c>
       <c r="B43" t="s">
         <v>4</v>
@@ -1077,12 +1083,12 @@
         <v>11</v>
       </c>
       <c r="D43" s="1">
-        <v>123</v>
+        <v>502</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="1">
-        <v>5075844</v>
+        <v>7215902</v>
       </c>
       <c r="B44" t="s">
         <v>4</v>
@@ -1091,12 +1097,12 @@
         <v>11</v>
       </c>
       <c r="D44" s="1">
-        <v>123</v>
+        <v>502</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="1">
-        <v>6889563</v>
+        <v>7200346</v>
       </c>
       <c r="B45" t="s">
         <v>4</v>
@@ -1105,158 +1111,158 @@
         <v>11</v>
       </c>
       <c r="D45" s="1">
-        <v>123</v>
+        <v>502</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="1">
-        <v>7346289</v>
+        <v>6307403</v>
       </c>
       <c r="B46" t="s">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D46" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1">
-        <v>7332471</v>
+        <v>3460035</v>
       </c>
       <c r="B47" t="s">
         <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D47" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="1">
-        <v>7330142</v>
+        <v>6944029</v>
       </c>
       <c r="B48" t="s">
         <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D48" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="1">
-        <v>3990488</v>
+        <v>7066399</v>
       </c>
       <c r="B49" t="s">
         <v>4</v>
       </c>
       <c r="C49" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D49" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="1">
-        <v>6998774</v>
+        <v>3540327</v>
       </c>
       <c r="B50" t="s">
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D50" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="1">
-        <v>7028014</v>
+        <v>7064865</v>
       </c>
       <c r="B51" t="s">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D51" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="1">
-        <v>7087009</v>
+        <v>3425893</v>
       </c>
       <c r="B52" t="s">
         <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D52" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="1">
-        <v>5816983</v>
+        <v>7397660</v>
       </c>
       <c r="B53" t="s">
         <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D53" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="1">
-        <v>7456256</v>
+        <v>7441525</v>
       </c>
       <c r="B54" t="s">
         <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D54" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="1">
-        <v>3269719</v>
+        <v>7206190</v>
       </c>
       <c r="B55" t="s">
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D55" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="1">
-        <v>7062720</v>
+        <v>5186353</v>
       </c>
       <c r="B56" t="s">
         <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D56" s="1">
         <v>123</v>
@@ -1264,97 +1270,97 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="1">
-        <v>7371352</v>
+        <v>7376836</v>
       </c>
       <c r="B57" t="s">
         <v>4</v>
       </c>
       <c r="C57" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D57" s="1">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="1">
-        <v>622192</v>
+        <v>7253979</v>
       </c>
       <c r="B58" t="s">
         <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D58" s="1">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="1">
-        <v>3194089</v>
+        <v>7577648</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D59" s="1">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="1">
-        <v>7275811</v>
+        <v>7197261</v>
       </c>
       <c r="B60" t="s">
         <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D60" s="1">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="1">
-        <v>3542596</v>
+        <v>7355494</v>
       </c>
       <c r="B61" t="s">
         <v>4</v>
       </c>
       <c r="C61" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D61" s="1">
-        <v>123</v>
+        <v>151</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="1">
-        <v>6081928</v>
+        <v>7262549</v>
       </c>
       <c r="B62" t="s">
         <v>4</v>
       </c>
       <c r="C62" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D62" s="1">
-        <v>123</v>
+        <v>151</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="1">
-        <v>7264983</v>
+        <v>7507621</v>
       </c>
       <c r="B63" t="s">
         <v>4</v>
       </c>
       <c r="C63" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D63" s="1">
         <v>151</v>
@@ -1362,13 +1368,13 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="1">
-        <v>3374411</v>
+        <v>6967656</v>
       </c>
       <c r="B64" t="s">
         <v>4</v>
       </c>
       <c r="C64" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D64" s="1">
         <v>151</v>
@@ -1376,405 +1382,405 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="1">
-        <v>6866204</v>
+        <v>641317</v>
       </c>
       <c r="B65" t="s">
         <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D65" s="1">
-        <v>151</v>
+        <v>801</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="1">
-        <v>4882381</v>
+        <v>6703284</v>
       </c>
       <c r="B66" t="s">
         <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D66" s="1">
-        <v>151</v>
+        <v>801</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="1">
-        <v>6010470</v>
+        <v>7094096</v>
       </c>
       <c r="B67" t="s">
         <v>4</v>
       </c>
       <c r="C67" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D67" s="1">
-        <v>406</v>
+        <v>801</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="1">
-        <v>6989424</v>
+        <v>6473441</v>
       </c>
       <c r="B68" t="s">
         <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D68" s="1">
-        <v>406</v>
+        <v>804</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="1">
-        <v>7229164</v>
+        <v>6569604</v>
       </c>
       <c r="B69" t="s">
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D69" s="1">
-        <v>406</v>
+        <v>804</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="1">
-        <v>1303951</v>
+        <v>6629393</v>
       </c>
       <c r="B70" t="s">
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D70" s="1">
-        <v>606</v>
+        <v>804</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="1">
-        <v>3497654</v>
+        <v>6673609</v>
       </c>
       <c r="B71" t="s">
         <v>4</v>
       </c>
       <c r="C71" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D71" s="1">
-        <v>606</v>
+        <v>804</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="1">
-        <v>5176468</v>
+        <v>7209637</v>
       </c>
       <c r="B72" t="s">
         <v>4</v>
       </c>
       <c r="C72" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D72" s="1">
-        <v>154</v>
+        <v>804</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="1">
-        <v>5446130</v>
+        <v>6825145</v>
       </c>
       <c r="B73" t="s">
         <v>4</v>
       </c>
       <c r="C73" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D73" s="1">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="1">
-        <v>5856071</v>
+        <v>7199072</v>
       </c>
       <c r="B74" t="s">
         <v>4</v>
       </c>
       <c r="C74" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D74" s="1">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="1">
-        <v>6187124</v>
+        <v>7577101</v>
       </c>
       <c r="B75" t="s">
         <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D75" s="1">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="1">
-        <v>6202390</v>
+        <v>7577022</v>
       </c>
       <c r="B76" t="s">
         <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D76" s="1">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="1">
-        <v>6555550</v>
+        <v>7460665</v>
       </c>
       <c r="B77" t="s">
         <v>4</v>
       </c>
       <c r="C77" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D77" s="1">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="1">
-        <v>7060208</v>
+        <v>6607068</v>
       </c>
       <c r="B78" t="s">
         <v>4</v>
       </c>
       <c r="C78" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D78" s="1">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="1">
-        <v>6995113</v>
+        <v>6954115</v>
       </c>
       <c r="B79" t="s">
         <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D79" s="1">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="1">
-        <v>6222515</v>
+        <v>5382299</v>
       </c>
       <c r="B80" t="s">
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D80" s="1">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="1">
-        <v>7537502</v>
+        <v>7513900</v>
       </c>
       <c r="B81" t="s">
         <v>4</v>
       </c>
       <c r="C81" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D81" s="1">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="1">
-        <v>7254410</v>
+        <v>6139260</v>
       </c>
       <c r="B82" t="s">
         <v>4</v>
       </c>
       <c r="C82" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D82" s="1">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="1">
-        <v>6427471</v>
+        <v>6982248</v>
       </c>
       <c r="B83" t="s">
         <v>4</v>
       </c>
       <c r="C83" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D83" s="1">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="1">
-        <v>6667522</v>
+        <v>7560014</v>
       </c>
       <c r="B84" t="s">
         <v>4</v>
       </c>
       <c r="C84" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D84" s="1">
-        <v>805</v>
+        <v>114</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="1">
-        <v>5688772</v>
+        <v>7375146</v>
       </c>
       <c r="B85" t="s">
         <v>4</v>
       </c>
       <c r="C85" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D85" s="1">
-        <v>805</v>
+        <v>114</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="1">
-        <v>7075120</v>
+        <v>6285090</v>
       </c>
       <c r="B86" t="s">
         <v>4</v>
       </c>
       <c r="C86" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D86" s="1">
-        <v>805</v>
+        <v>604</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="1">
-        <v>5692718</v>
+        <v>3055103</v>
       </c>
       <c r="B87" t="s">
         <v>4</v>
       </c>
       <c r="C87" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D87" s="1">
-        <v>805</v>
+        <v>604</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="1">
-        <v>3450142</v>
+        <v>7457647</v>
       </c>
       <c r="B88" t="s">
         <v>4</v>
       </c>
       <c r="C88" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D88" s="1">
-        <v>805</v>
+        <v>604</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="1">
-        <v>7483348</v>
+        <v>6270833</v>
       </c>
       <c r="B89" t="s">
         <v>4</v>
       </c>
       <c r="C89" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D89" s="1">
-        <v>805</v>
+        <v>307</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="1">
-        <v>6567826</v>
+        <v>6410802</v>
       </c>
       <c r="B90" t="s">
         <v>4</v>
       </c>
       <c r="C90" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D90" s="1">
-        <v>805</v>
+        <v>307</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="1">
-        <v>6181545</v>
+        <v>7510353</v>
       </c>
       <c r="B91" t="s">
         <v>4</v>
       </c>
       <c r="C91" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D91" s="1">
-        <v>805</v>
+        <v>307</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="1">
-        <v>5465632</v>
+        <v>7235596</v>
       </c>
       <c r="B92" t="s">
         <v>4</v>
       </c>
       <c r="C92" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D92" s="1">
-        <v>805</v>
+        <v>307</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="1">
-        <v>6410832</v>
+        <v>2878257</v>
       </c>
       <c r="B93" t="s">
         <v>4</v>
       </c>
       <c r="C93" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D93" s="1">
         <v>307</v>
@@ -1782,13 +1788,13 @@
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="1">
-        <v>6219111</v>
+        <v>7500702</v>
       </c>
       <c r="B94" t="s">
         <v>4</v>
       </c>
       <c r="C94" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D94" s="1">
         <v>307</v>
@@ -1796,13 +1802,13 @@
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="1">
-        <v>2069609</v>
+        <v>6344857</v>
       </c>
       <c r="B95" t="s">
         <v>4</v>
       </c>
       <c r="C95" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D95" s="1">
         <v>307</v>
@@ -1810,469 +1816,469 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="1">
-        <v>3179797</v>
+        <v>5510670</v>
       </c>
       <c r="B96" t="s">
         <v>4</v>
       </c>
       <c r="C96" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D96" s="1">
-        <v>307</v>
+        <v>603</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="1">
-        <v>7212659</v>
+        <v>6221599</v>
       </c>
       <c r="B97" t="s">
         <v>4</v>
       </c>
       <c r="C97" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D97" s="1">
-        <v>307</v>
+        <v>505</v>
       </c>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="1">
-        <v>7500045</v>
+        <v>5538095</v>
       </c>
       <c r="B98" t="s">
         <v>4</v>
       </c>
       <c r="C98" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D98" s="1">
-        <v>603</v>
+        <v>505</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="1">
-        <v>7506597</v>
+        <v>5455252</v>
       </c>
       <c r="B99" t="s">
         <v>4</v>
       </c>
       <c r="C99" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D99" s="1">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="1">
-        <v>2470543</v>
+        <v>6285788</v>
       </c>
       <c r="B100" t="s">
         <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D100" s="1">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="1">
-        <v>5172148</v>
+        <v>5181870</v>
       </c>
       <c r="B101" t="s">
         <v>4</v>
       </c>
       <c r="C101" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D101" s="1">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="1">
-        <v>7248275</v>
+        <v>6601032</v>
       </c>
       <c r="B102" t="s">
         <v>4</v>
       </c>
       <c r="C102" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D102" s="1">
-        <v>803</v>
+        <v>505</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="1">
-        <v>7349586</v>
+        <v>7068453</v>
       </c>
       <c r="B103" t="s">
         <v>4</v>
       </c>
       <c r="C103" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D103" s="1">
-        <v>803</v>
+        <v>505</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="1">
-        <v>7076629</v>
+        <v>3497654</v>
       </c>
       <c r="B104" t="s">
         <v>4</v>
       </c>
       <c r="C104" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D104" s="1">
-        <v>803</v>
+        <v>606</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="1">
-        <v>7560495</v>
+        <v>5891561</v>
       </c>
       <c r="B105" t="s">
         <v>4</v>
       </c>
       <c r="C105" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D105" s="1">
-        <v>803</v>
+        <v>805</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="1">
-        <v>7079974</v>
+        <v>6968628</v>
       </c>
       <c r="B106" t="s">
         <v>4</v>
       </c>
       <c r="C106" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D106" s="1">
-        <v>803</v>
+        <v>805</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="1">
-        <v>7462843</v>
+        <v>5230228</v>
       </c>
       <c r="B107" t="s">
         <v>4</v>
       </c>
       <c r="C107" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D107" s="1">
-        <v>803</v>
+        <v>805</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="1">
-        <v>3959813</v>
+        <v>6569618</v>
       </c>
       <c r="B108" t="s">
         <v>4</v>
       </c>
       <c r="C108" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D108" s="1">
-        <v>152</v>
+        <v>805</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="1">
-        <v>7532811</v>
+        <v>4741123</v>
       </c>
       <c r="B109" t="s">
         <v>4</v>
       </c>
       <c r="C109" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D109" s="1">
-        <v>152</v>
+        <v>805</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="1">
-        <v>7063212</v>
+        <v>7525177</v>
       </c>
       <c r="B110" t="s">
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D110" s="1">
-        <v>152</v>
+        <v>805</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="1">
-        <v>5722898</v>
+        <v>6567826</v>
       </c>
       <c r="B111" t="s">
         <v>4</v>
       </c>
       <c r="C111" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D111" s="1">
-        <v>605</v>
+        <v>805</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="1">
-        <v>5714504</v>
+        <v>7075120</v>
       </c>
       <c r="B112" t="s">
         <v>4</v>
       </c>
       <c r="C112" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D112" s="1">
-        <v>605</v>
+        <v>805</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="1">
-        <v>51750954</v>
+        <v>7359806</v>
       </c>
       <c r="B113" t="s">
         <v>4</v>
       </c>
       <c r="C113" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D113" s="1">
-        <v>506</v>
+        <v>805</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="1">
-        <v>5885294</v>
+        <v>7032346</v>
       </c>
       <c r="B114" t="s">
         <v>4</v>
       </c>
       <c r="C114" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="D114" s="1">
-        <v>502</v>
+        <v>805</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="1">
-        <v>4480229</v>
+        <v>7422485</v>
       </c>
       <c r="B115" t="s">
         <v>4</v>
       </c>
       <c r="C115" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D115" s="1">
-        <v>140</v>
+        <v>805</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="1">
-        <v>4402003</v>
+        <v>6181545</v>
       </c>
       <c r="B116" t="s">
         <v>4</v>
       </c>
       <c r="C116" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D116" s="1">
-        <v>140</v>
+        <v>805</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="1">
-        <v>3216471</v>
+        <v>7060208</v>
       </c>
       <c r="B117" t="s">
         <v>4</v>
       </c>
       <c r="C117" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D117" s="1">
-        <v>140</v>
+        <v>805</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="1">
-        <v>5851002</v>
+        <v>7215889</v>
       </c>
       <c r="B118" t="s">
         <v>4</v>
       </c>
       <c r="C118" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D118" s="1">
-        <v>140</v>
+        <v>803</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="1">
-        <v>6280939</v>
+        <v>67689098</v>
       </c>
       <c r="B119" t="s">
         <v>4</v>
       </c>
       <c r="C119" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D119" s="1">
-        <v>140</v>
+        <v>803</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="1">
-        <v>6145956</v>
+        <v>6047324</v>
       </c>
       <c r="B120" t="s">
         <v>4</v>
       </c>
       <c r="C120" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D120" s="1">
-        <v>503</v>
+        <v>803</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="1">
-        <v>7480709</v>
+        <v>7525440</v>
       </c>
       <c r="B121" t="s">
         <v>4</v>
       </c>
       <c r="C121" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D121" s="1">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="1">
-        <v>6887014</v>
+        <v>7228558</v>
       </c>
       <c r="B122" t="s">
         <v>4</v>
       </c>
       <c r="C122" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D122" s="1">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="1">
-        <v>6570809</v>
+        <v>6931087</v>
       </c>
       <c r="B123" t="s">
         <v>4</v>
       </c>
       <c r="C123" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D123" s="1">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="1">
-        <v>2539133</v>
+        <v>4778297</v>
       </c>
       <c r="B124" t="s">
         <v>4</v>
       </c>
       <c r="C124" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D124" s="1">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="1">
-        <v>3426581</v>
+        <v>600960</v>
       </c>
       <c r="B125" t="s">
         <v>4</v>
       </c>
       <c r="C125" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D125" s="1">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="1">
-        <v>5110749</v>
+        <v>7344978</v>
       </c>
       <c r="B126" t="s">
         <v>4</v>
       </c>
       <c r="C126" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D126" s="1">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="1">
-        <v>6020204</v>
+        <v>6277523</v>
       </c>
       <c r="B127" t="s">
         <v>4</v>
       </c>
       <c r="C127" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D127" s="1">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="1">
-        <v>7104711</v>
+        <v>3428583</v>
       </c>
       <c r="B128" t="s">
         <v>4</v>
       </c>
       <c r="C128" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D128" s="1">
-        <v>603</v>
+        <v>803</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="1">
-        <v>7235340</v>
+        <v>7576713</v>
       </c>
       <c r="B129" t="s">
         <v>4</v>
@@ -2281,82 +2287,82 @@
         <v>26</v>
       </c>
       <c r="D129" s="1">
-        <v>134</v>
+        <v>803</v>
       </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="1">
-        <v>6474838</v>
+        <v>3426581</v>
       </c>
       <c r="B130" t="s">
         <v>4</v>
       </c>
       <c r="C130" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D130" s="1">
-        <v>134</v>
+        <v>804</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="1">
-        <v>7441501</v>
+        <v>7289995</v>
       </c>
       <c r="B131" t="s">
         <v>4</v>
       </c>
       <c r="C131" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D131" s="1">
-        <v>134</v>
+        <v>804</v>
       </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="1">
-        <v>3267158</v>
+        <v>7259213</v>
       </c>
       <c r="B132" t="s">
         <v>4</v>
       </c>
       <c r="C132" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D132" s="1">
-        <v>134</v>
+        <v>603</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="1">
-        <v>7395571</v>
+        <v>653294</v>
       </c>
       <c r="B133" t="s">
         <v>4</v>
       </c>
       <c r="C133" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D133" s="1">
-        <v>134</v>
+        <v>802</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="1">
-        <v>6931726</v>
+        <v>3391445</v>
       </c>
       <c r="B134" t="s">
         <v>4</v>
       </c>
       <c r="C134" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D134" s="1">
-        <v>134</v>
+        <v>801</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="1">
-        <v>7063237</v>
+        <v>5252010</v>
       </c>
       <c r="B135" t="s">
         <v>4</v>
@@ -2365,390 +2371,390 @@
         <v>27</v>
       </c>
       <c r="D135" s="1">
-        <v>604</v>
+        <v>506</v>
       </c>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="1">
-        <v>6187779</v>
+        <v>7483745</v>
       </c>
       <c r="B136" t="s">
         <v>4</v>
       </c>
       <c r="C136" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D136" s="1">
-        <v>503</v>
+        <v>506</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="1">
-        <v>6187781</v>
+        <v>6797299</v>
       </c>
       <c r="B137" t="s">
         <v>4</v>
       </c>
       <c r="C137" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D137" s="1">
-        <v>503</v>
+        <v>403</v>
       </c>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="1">
-        <v>5400149</v>
+        <v>3373822</v>
       </c>
       <c r="B138" t="s">
         <v>4</v>
       </c>
       <c r="C138" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D138" s="1">
-        <v>503</v>
+        <v>403</v>
       </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="1">
-        <v>7254228</v>
+        <v>3450004</v>
       </c>
       <c r="B139" t="s">
         <v>4</v>
       </c>
       <c r="C139" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D139" s="1">
-        <v>503</v>
+        <v>403</v>
       </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="1">
-        <v>7552795</v>
+        <v>6810964</v>
       </c>
       <c r="B140" t="s">
         <v>4</v>
       </c>
       <c r="C140" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D140" s="1">
-        <v>503</v>
+        <v>406</v>
       </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="1">
-        <v>5432669</v>
+        <v>4054442</v>
       </c>
       <c r="B141" t="s">
         <v>4</v>
       </c>
       <c r="C141" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D141" s="1">
-        <v>503</v>
+        <v>406</v>
       </c>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="1">
-        <v>6787781</v>
+        <v>3492270</v>
       </c>
       <c r="B142" t="s">
         <v>4</v>
       </c>
       <c r="C142" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D142" s="1">
-        <v>503</v>
+        <v>406</v>
       </c>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="1">
-        <v>9443388</v>
+        <v>7040001</v>
       </c>
       <c r="B143" t="s">
         <v>4</v>
       </c>
       <c r="C143" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D143" s="1">
-        <v>504</v>
+        <v>407</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="1">
-        <v>7051183</v>
+        <v>7230030</v>
       </c>
       <c r="B144" t="s">
         <v>4</v>
       </c>
       <c r="C144" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D144" s="1">
-        <v>504</v>
+        <v>407</v>
       </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="1">
-        <v>7539210</v>
+        <v>7202350</v>
       </c>
       <c r="B145" t="s">
         <v>4</v>
       </c>
       <c r="C145" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D145" s="1">
-        <v>504</v>
+        <v>308</v>
       </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="1">
-        <v>7554748</v>
+        <v>7240100</v>
       </c>
       <c r="B146" t="s">
         <v>4</v>
       </c>
       <c r="C146" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D146" s="1">
-        <v>504</v>
+        <v>308</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="1">
-        <v>1882576</v>
+        <v>5029711</v>
       </c>
       <c r="B147" t="s">
         <v>4</v>
       </c>
       <c r="C147" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D147" s="1">
-        <v>504</v>
+        <v>308</v>
       </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="1">
-        <v>5593493</v>
+        <v>3062209</v>
       </c>
       <c r="B148" t="s">
         <v>4</v>
       </c>
       <c r="C148" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D148" s="1">
-        <v>504</v>
+        <v>308</v>
       </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="1">
-        <v>7466007</v>
+        <v>3427111</v>
       </c>
       <c r="B149" t="s">
         <v>4</v>
       </c>
       <c r="C149" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D149" s="1">
-        <v>504</v>
+        <v>308</v>
       </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="1">
-        <v>5460701</v>
+        <v>6978244</v>
       </c>
       <c r="B150" t="s">
         <v>4</v>
       </c>
       <c r="C150" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D150" s="1">
-        <v>504</v>
+        <v>308</v>
       </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="1">
-        <v>5178875</v>
+        <v>7038664</v>
       </c>
       <c r="B151" t="s">
         <v>4</v>
       </c>
       <c r="C151" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D151" s="1">
-        <v>504</v>
+        <v>308</v>
       </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="1">
-        <v>5175541</v>
+        <v>6091016</v>
       </c>
       <c r="B152" t="s">
         <v>4</v>
       </c>
       <c r="C152" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D152" s="1">
-        <v>504</v>
+        <v>602</v>
       </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="1">
-        <v>5603147</v>
+        <v>7023240</v>
       </c>
       <c r="B153" t="s">
         <v>4</v>
       </c>
       <c r="C153" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D153" s="1">
-        <v>504</v>
+        <v>605</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="1">
-        <v>7025924</v>
+        <v>3059109</v>
       </c>
       <c r="B154" t="s">
         <v>4</v>
       </c>
       <c r="C154" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D154" s="1">
-        <v>504</v>
+        <v>201</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="1">
-        <v>7537382</v>
+        <v>7212855</v>
       </c>
       <c r="B155" t="s">
         <v>4</v>
       </c>
       <c r="C155" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D155" s="1">
-        <v>504</v>
+        <v>201</v>
       </c>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="1">
-        <v>7545927</v>
+        <v>6705285</v>
       </c>
       <c r="B156" t="s">
         <v>4</v>
       </c>
       <c r="C156" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D156" s="1">
-        <v>504</v>
+        <v>201</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="1">
-        <v>7017743</v>
+        <v>7409656</v>
       </c>
       <c r="B157" t="s">
         <v>4</v>
       </c>
       <c r="C157" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D157" s="1">
-        <v>504</v>
+        <v>201</v>
       </c>
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="1">
-        <v>6266859</v>
+        <v>6949619</v>
       </c>
       <c r="B158" t="s">
         <v>4</v>
       </c>
       <c r="C158" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D158" s="1">
-        <v>404</v>
+        <v>201</v>
       </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="1">
-        <v>7422454</v>
+        <v>5872977</v>
       </c>
       <c r="B159" t="s">
         <v>4</v>
       </c>
       <c r="C159" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D159" s="1">
-        <v>404</v>
+        <v>504</v>
       </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="1">
-        <v>6095823</v>
+        <v>7545927</v>
       </c>
       <c r="B160" t="s">
         <v>4</v>
       </c>
       <c r="C160" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D160" s="1">
-        <v>404</v>
+        <v>504</v>
       </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="1">
-        <v>3499292</v>
+        <v>5170837</v>
       </c>
       <c r="B161" t="s">
         <v>4</v>
       </c>
       <c r="C161" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D161" s="1">
-        <v>404</v>
+        <v>504</v>
       </c>
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="1">
-        <v>6159707</v>
+        <v>5172744</v>
       </c>
       <c r="B162" t="s">
         <v>4</v>
       </c>
       <c r="C162" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D162" s="1">
-        <v>404</v>
+        <v>504</v>
       </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="1">
-        <v>7069075</v>
+        <v>5817316</v>
       </c>
       <c r="B163" t="s">
         <v>4</v>
@@ -2757,77 +2763,217 @@
         <v>29</v>
       </c>
       <c r="D163" s="1">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="1">
-        <v>6959769</v>
+        <v>924017</v>
       </c>
       <c r="B164" t="s">
         <v>4</v>
       </c>
       <c r="C164" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="D164" s="1">
-        <v>404</v>
+        <v>123</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="1">
-        <v>7339861</v>
+        <v>7206189</v>
       </c>
       <c r="B165" t="s">
         <v>4</v>
       </c>
       <c r="C165" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D165" s="1">
-        <v>133</v>
+        <v>123</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="1">
-        <v>7373767</v>
+        <v>3064665</v>
       </c>
       <c r="B166" t="s">
         <v>4</v>
       </c>
       <c r="C166" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D166" s="1">
-        <v>133</v>
+        <v>123</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="1">
-        <v>6553655</v>
+        <v>7055133</v>
       </c>
       <c r="B167" t="s">
         <v>4</v>
       </c>
       <c r="C167" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="D167" s="1">
-        <v>403</v>
+        <v>123</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="1">
-        <v>2955535</v>
+        <v>7064958</v>
       </c>
       <c r="B168" t="s">
         <v>4</v>
       </c>
       <c r="C168" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="D168" s="1">
-        <v>201</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4">
+      <c r="A169" s="1">
+        <v>3990488</v>
+      </c>
+      <c r="B169" t="s">
+        <v>4</v>
+      </c>
+      <c r="C169" t="s">
+        <v>13</v>
+      </c>
+      <c r="D169" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4">
+      <c r="A170" s="1">
+        <v>5075844</v>
+      </c>
+      <c r="B170" t="s">
+        <v>4</v>
+      </c>
+      <c r="C170" t="s">
+        <v>13</v>
+      </c>
+      <c r="D170" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4">
+      <c r="A171" s="1">
+        <v>7346289</v>
+      </c>
+      <c r="B171" t="s">
+        <v>4</v>
+      </c>
+      <c r="C171" t="s">
+        <v>13</v>
+      </c>
+      <c r="D171" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4">
+      <c r="A172" s="1">
+        <v>7031864</v>
+      </c>
+      <c r="B172" t="s">
+        <v>4</v>
+      </c>
+      <c r="C172" t="s">
+        <v>13</v>
+      </c>
+      <c r="D172" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4">
+      <c r="A173" s="1">
+        <v>5420681</v>
+      </c>
+      <c r="B173" t="s">
+        <v>4</v>
+      </c>
+      <c r="C173" t="s">
+        <v>13</v>
+      </c>
+      <c r="D173" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4">
+      <c r="A174" s="1">
+        <v>6908570</v>
+      </c>
+      <c r="B174" t="s">
+        <v>4</v>
+      </c>
+      <c r="C174" t="s">
+        <v>13</v>
+      </c>
+      <c r="D174" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4">
+      <c r="A175" s="1">
+        <v>7022850</v>
+      </c>
+      <c r="B175" t="s">
+        <v>4</v>
+      </c>
+      <c r="C175" t="s">
+        <v>13</v>
+      </c>
+      <c r="D175" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4">
+      <c r="A176" s="1">
+        <v>6998774</v>
+      </c>
+      <c r="B176" t="s">
+        <v>4</v>
+      </c>
+      <c r="C176" t="s">
+        <v>13</v>
+      </c>
+      <c r="D176" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4">
+      <c r="A177" s="1">
+        <v>3392842</v>
+      </c>
+      <c r="B177" t="s">
+        <v>4</v>
+      </c>
+      <c r="C177" t="s">
+        <v>13</v>
+      </c>
+      <c r="D177" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4">
+      <c r="A178" s="1">
+        <v>6794062</v>
+      </c>
+      <c r="B178" t="s">
+        <v>4</v>
+      </c>
+      <c r="C178" t="s">
+        <v>13</v>
+      </c>
+      <c r="D178" s="1">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correção do código Novo automatizar_vendas.py, que estava apresentando falhas devido a atualização do whatsapp web
</commit_message>
<xml_diff>
--- a/Vendas_Do_Dia.xlsx
+++ b/Vendas_Do_Dia.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="39">
   <si>
     <t>Código</t>
   </si>
@@ -28,97 +28,109 @@
     <t>Código_Vendedor</t>
   </si>
   <si>
-    <t>18/03/2026</t>
+    <t>26/03/2026</t>
+  </si>
+  <si>
+    <t>Kenia</t>
+  </si>
+  <si>
+    <t>Caio Edson</t>
+  </si>
+  <si>
+    <t>Camilo</t>
+  </si>
+  <si>
+    <t>Bruno</t>
+  </si>
+  <si>
+    <t>Sebastião</t>
+  </si>
+  <si>
+    <t>Jose Jose Vicente</t>
+  </si>
+  <si>
+    <t>Narjara</t>
+  </si>
+  <si>
+    <t>Suene</t>
+  </si>
+  <si>
+    <t>Lorrane</t>
+  </si>
+  <si>
+    <t>Manoel</t>
+  </si>
+  <si>
+    <t>Janaína</t>
+  </si>
+  <si>
+    <t>Ian</t>
+  </si>
+  <si>
+    <t>Álvaro</t>
+  </si>
+  <si>
+    <t>Marcão</t>
+  </si>
+  <si>
+    <t>Wellinton</t>
+  </si>
+  <si>
+    <t>Robson</t>
   </si>
   <si>
     <t>Marcos Vinicius</t>
   </si>
   <si>
+    <t>Aurélio</t>
+  </si>
+  <si>
+    <t>Victor Pereira</t>
+  </si>
+  <si>
     <t>Jerques</t>
   </si>
   <si>
-    <t>Sebastião</t>
+    <t>Leandro</t>
+  </si>
+  <si>
+    <t>Luis Felipe</t>
+  </si>
+  <si>
+    <t>Maycon</t>
+  </si>
+  <si>
+    <t>Guilherme</t>
+  </si>
+  <si>
+    <t>Larissa</t>
+  </si>
+  <si>
+    <t>Filipe Assis</t>
   </si>
   <si>
     <t>Michel</t>
   </si>
   <si>
-    <t>Caíque Mansur</t>
-  </si>
-  <si>
-    <t>Kenia</t>
-  </si>
-  <si>
-    <t>Filipe Assis</t>
-  </si>
-  <si>
-    <t>Ian</t>
-  </si>
-  <si>
-    <t>Suene</t>
-  </si>
-  <si>
-    <t>Camilo</t>
-  </si>
-  <si>
-    <t>Álvaro</t>
-  </si>
-  <si>
-    <t>Victor Prazeres</t>
+    <t>Daniele</t>
   </si>
   <si>
     <t>Davidson</t>
   </si>
   <si>
-    <t>Lorrane</t>
-  </si>
-  <si>
-    <t>Narjara</t>
+    <t>Mateus</t>
+  </si>
+  <si>
+    <t>Alexandre</t>
+  </si>
+  <si>
+    <t>Cadu</t>
+  </si>
+  <si>
+    <t>Ana Luiza</t>
   </si>
   <si>
     <t>Monique</t>
-  </si>
-  <si>
-    <t>Guilherme</t>
-  </si>
-  <si>
-    <t>Ana Luiza</t>
-  </si>
-  <si>
-    <t>Luis Felipe</t>
-  </si>
-  <si>
-    <t>Victor Pereira</t>
-  </si>
-  <si>
-    <t>Wellinton</t>
-  </si>
-  <si>
-    <t>Aurélio</t>
-  </si>
-  <si>
-    <t>Paulo</t>
-  </si>
-  <si>
-    <t>Robson</t>
-  </si>
-  <si>
-    <t>Maycon</t>
-  </si>
-  <si>
-    <t>Alisson</t>
-  </si>
-  <si>
-    <t>Bruno</t>
-  </si>
-  <si>
-    <t>Caio Edson</t>
-  </si>
-  <si>
-    <t>Daniele</t>
-  </si>
-  <si>
-    <t>Alexandre</t>
   </si>
 </sst>
 </file>
@@ -477,10 +489,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D178"/>
+  <dimension ref="A1:D220"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="35.7109375" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -500,7 +514,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1">
-        <v>6560577</v>
+        <v>1214626</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -509,68 +523,68 @@
         <v>5</v>
       </c>
       <c r="D2" s="1">
-        <v>404</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1">
-        <v>6938561</v>
+        <v>2096604</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="1">
-        <v>404</v>
+        <v>605</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1">
-        <v>6023751</v>
+        <v>2864493</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1">
-        <v>404</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1">
-        <v>7535398</v>
+        <v>2895839</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D5" s="1">
-        <v>404</v>
+        <v>602</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1">
-        <v>5976217</v>
+        <v>2955045</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D6" s="1">
-        <v>308</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1">
-        <v>6933444</v>
+        <v>2961677</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
@@ -579,116 +593,116 @@
         <v>7</v>
       </c>
       <c r="D7" s="1">
-        <v>401</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1">
-        <v>3664967</v>
+        <v>2963164</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1">
-        <v>401</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1">
-        <v>5398731</v>
+        <v>3056028</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D9" s="1">
-        <v>401</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1">
-        <v>7576963</v>
+        <v>3058330</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D10" s="1">
-        <v>401</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1">
-        <v>3290202</v>
+        <v>3058469</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D11" s="1">
-        <v>401</v>
+        <v>802</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1">
-        <v>3324270</v>
+        <v>3191550</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D12" s="1">
-        <v>401</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1">
-        <v>6962447</v>
+        <v>3368361</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D13" s="1">
-        <v>401</v>
+        <v>405</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1">
-        <v>6929705</v>
+        <v>3390409</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D14" s="1">
-        <v>401</v>
+        <v>503</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1">
-        <v>7409406</v>
+        <v>3428236</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D15" s="1">
         <v>401</v>
@@ -696,147 +710,147 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1">
-        <v>3452176</v>
+        <v>3483281</v>
       </c>
       <c r="B16" t="s">
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D16" s="1">
-        <v>401</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1">
-        <v>3331471</v>
+        <v>3487804</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D17" s="1">
-        <v>401</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="1">
-        <v>6954098</v>
+        <v>3536216</v>
       </c>
       <c r="B18" t="s">
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D18" s="1">
-        <v>401</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1">
-        <v>7332052</v>
+        <v>3561484</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D19" s="1">
-        <v>401</v>
+        <v>151</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1">
-        <v>7568265</v>
+        <v>3584689</v>
       </c>
       <c r="B20" t="s">
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D20" s="1">
-        <v>401</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1">
-        <v>652507</v>
+        <v>3636164</v>
       </c>
       <c r="B21" t="s">
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D21" s="1">
-        <v>402</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1">
-        <v>2903112</v>
+        <v>3685541</v>
       </c>
       <c r="B22" t="s">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D22" s="1">
-        <v>402</v>
+        <v>805</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1">
-        <v>3587027</v>
+        <v>3739153</v>
       </c>
       <c r="B23" t="s">
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D23" s="1">
-        <v>402</v>
+        <v>605</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="1">
-        <v>6562716</v>
+        <v>3742998</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D24" s="1">
-        <v>402</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1">
-        <v>3215539</v>
+        <v>3768054</v>
       </c>
       <c r="B25" t="s">
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D25" s="1">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="1">
-        <v>6260739</v>
+        <v>3798542</v>
       </c>
       <c r="B26" t="s">
         <v>4</v>
@@ -845,208 +859,208 @@
         <v>8</v>
       </c>
       <c r="D26" s="1">
-        <v>402</v>
+        <v>602</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="1">
-        <v>7523946</v>
+        <v>3847552</v>
       </c>
       <c r="B27" t="s">
         <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D27" s="1">
-        <v>402</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="1">
-        <v>5729276</v>
+        <v>3954392</v>
       </c>
       <c r="B28" t="s">
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D28" s="1">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="1">
-        <v>7288549</v>
+        <v>3990488</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D29" s="1">
-        <v>150</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="1">
-        <v>6459199</v>
+        <v>4055631</v>
       </c>
       <c r="B30" t="s">
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D30" s="1">
-        <v>134</v>
+        <v>803</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1">
-        <v>4993036</v>
+        <v>4060534</v>
       </c>
       <c r="B31" t="s">
         <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D31" s="1">
-        <v>134</v>
+        <v>405</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1">
-        <v>6121904</v>
+        <v>4136116</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
       </c>
       <c r="C32" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D32" s="1">
-        <v>134</v>
+        <v>805</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1">
-        <v>6703859</v>
+        <v>4271763</v>
       </c>
       <c r="B33" t="s">
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D33" s="1">
-        <v>134</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1">
-        <v>6802435</v>
+        <v>4350215</v>
       </c>
       <c r="B34" t="s">
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D34" s="1">
-        <v>134</v>
+        <v>405</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1">
-        <v>6752243</v>
+        <v>4778292</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D35" s="1">
-        <v>134</v>
+        <v>803</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1">
-        <v>7396713</v>
+        <v>4869849</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D36" s="1">
-        <v>308</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="1">
-        <v>2850271</v>
+        <v>4936753</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D37" s="1">
-        <v>308</v>
+        <v>805</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1">
-        <v>7066398</v>
+        <v>5077402</v>
       </c>
       <c r="B38" t="s">
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D38" s="1">
-        <v>502</v>
+        <v>605</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1">
-        <v>6163577</v>
+        <v>5134863</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D39" s="1">
-        <v>502</v>
+        <v>606</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1">
-        <v>7288831</v>
+        <v>5159677</v>
       </c>
       <c r="B40" t="s">
         <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D40" s="1">
-        <v>502</v>
+        <v>308</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1">
-        <v>7553536</v>
+        <v>5163170</v>
       </c>
       <c r="B41" t="s">
         <v>4</v>
@@ -1055,320 +1069,320 @@
         <v>11</v>
       </c>
       <c r="D41" s="1">
-        <v>502</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="1">
-        <v>7236527</v>
+        <v>5169133</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D42" s="1">
-        <v>502</v>
+        <v>807</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1">
-        <v>7522960</v>
+        <v>5171245</v>
       </c>
       <c r="B43" t="s">
         <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D43" s="1">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="1">
-        <v>7215902</v>
+        <v>5172155</v>
       </c>
       <c r="B44" t="s">
         <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D44" s="1">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="1">
-        <v>7200346</v>
+        <v>5172158</v>
       </c>
       <c r="B45" t="s">
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D45" s="1">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="1">
-        <v>6307403</v>
+        <v>5172254</v>
       </c>
       <c r="B46" t="s">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D46" s="1">
-        <v>301</v>
+        <v>405</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1">
-        <v>3460035</v>
+        <v>5181659</v>
       </c>
       <c r="B47" t="s">
         <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D47" s="1">
-        <v>301</v>
+        <v>505</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="1">
-        <v>6944029</v>
+        <v>5181870</v>
       </c>
       <c r="B48" t="s">
         <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D48" s="1">
-        <v>301</v>
+        <v>505</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="1">
-        <v>7066399</v>
+        <v>5244562</v>
       </c>
       <c r="B49" t="s">
         <v>4</v>
       </c>
       <c r="C49" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="D49" s="1">
-        <v>301</v>
+        <v>406</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="1">
-        <v>3540327</v>
+        <v>5302610</v>
       </c>
       <c r="B50" t="s">
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D50" s="1">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="1">
-        <v>7064865</v>
+        <v>5335575</v>
       </c>
       <c r="B51" t="s">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="D51" s="1">
-        <v>301</v>
+        <v>501</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="1">
-        <v>3425893</v>
+        <v>5345375</v>
       </c>
       <c r="B52" t="s">
         <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="D52" s="1">
-        <v>301</v>
+        <v>501</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="1">
-        <v>7397660</v>
+        <v>5351260</v>
       </c>
       <c r="B53" t="s">
         <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D53" s="1">
-        <v>301</v>
+        <v>502</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="1">
-        <v>7441525</v>
+        <v>5352620</v>
       </c>
       <c r="B54" t="s">
         <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="D54" s="1">
-        <v>301</v>
+        <v>501</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="1">
-        <v>7206190</v>
+        <v>5353720</v>
       </c>
       <c r="B55" t="s">
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D55" s="1">
-        <v>301</v>
+        <v>119</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="1">
-        <v>5186353</v>
+        <v>5365641</v>
       </c>
       <c r="B56" t="s">
         <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D56" s="1">
-        <v>123</v>
+        <v>501</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="1">
-        <v>7376836</v>
+        <v>5369534</v>
       </c>
       <c r="B57" t="s">
         <v>4</v>
       </c>
       <c r="C57" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D57" s="1">
-        <v>133</v>
+        <v>151</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="1">
-        <v>7253979</v>
+        <v>5389856</v>
       </c>
       <c r="B58" t="s">
         <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D58" s="1">
-        <v>133</v>
+        <v>802</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="1">
-        <v>7577648</v>
+        <v>5398157</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D59" s="1">
-        <v>133</v>
+        <v>503</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="1">
-        <v>7197261</v>
+        <v>5413877</v>
       </c>
       <c r="B60" t="s">
         <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D60" s="1">
-        <v>133</v>
+        <v>501</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="1">
-        <v>7355494</v>
+        <v>5416788</v>
       </c>
       <c r="B61" t="s">
         <v>4</v>
       </c>
       <c r="C61" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D61" s="1">
-        <v>151</v>
+        <v>501</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="1">
-        <v>7262549</v>
+        <v>5419961</v>
       </c>
       <c r="B62" t="s">
         <v>4</v>
       </c>
       <c r="C62" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D62" s="1">
-        <v>151</v>
+        <v>134</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="1">
-        <v>7507621</v>
+        <v>5422561</v>
       </c>
       <c r="B63" t="s">
         <v>4</v>
       </c>
       <c r="C63" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D63" s="1">
-        <v>151</v>
+        <v>501</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="1">
-        <v>6967656</v>
+        <v>5430314</v>
       </c>
       <c r="B64" t="s">
         <v>4</v>
@@ -1377,130 +1391,130 @@
         <v>15</v>
       </c>
       <c r="D64" s="1">
-        <v>151</v>
+        <v>503</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="1">
-        <v>641317</v>
+        <v>5479878</v>
       </c>
       <c r="B65" t="s">
         <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D65" s="1">
-        <v>801</v>
+        <v>403</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="1">
-        <v>6703284</v>
+        <v>5482687</v>
       </c>
       <c r="B66" t="s">
         <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D66" s="1">
-        <v>801</v>
+        <v>404</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="1">
-        <v>7094096</v>
+        <v>5659006</v>
       </c>
       <c r="B67" t="s">
         <v>4</v>
       </c>
       <c r="C67" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D67" s="1">
-        <v>801</v>
+        <v>605</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="1">
-        <v>6473441</v>
+        <v>5727378</v>
       </c>
       <c r="B68" t="s">
         <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D68" s="1">
-        <v>804</v>
+        <v>402</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="1">
-        <v>6569604</v>
+        <v>5913508</v>
       </c>
       <c r="B69" t="s">
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D69" s="1">
-        <v>804</v>
+        <v>301</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="1">
-        <v>6629393</v>
+        <v>5989794</v>
       </c>
       <c r="B70" t="s">
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D70" s="1">
-        <v>804</v>
+        <v>119</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="1">
-        <v>6673609</v>
+        <v>6016194</v>
       </c>
       <c r="B71" t="s">
         <v>4</v>
       </c>
       <c r="C71" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="D71" s="1">
-        <v>804</v>
+        <v>201</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="1">
-        <v>7209637</v>
+        <v>6017477</v>
       </c>
       <c r="B72" t="s">
         <v>4</v>
       </c>
       <c r="C72" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D72" s="1">
-        <v>804</v>
+        <v>308</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="1">
-        <v>6825145</v>
+        <v>6020204</v>
       </c>
       <c r="B73" t="s">
         <v>4</v>
       </c>
       <c r="C73" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D73" s="1">
         <v>804</v>
@@ -1508,307 +1522,307 @@
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="1">
-        <v>7199072</v>
+        <v>6036625</v>
       </c>
       <c r="B74" t="s">
         <v>4</v>
       </c>
       <c r="C74" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D74" s="1">
-        <v>804</v>
+        <v>308</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="1">
-        <v>7577101</v>
+        <v>6047728</v>
       </c>
       <c r="B75" t="s">
         <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="D75" s="1">
-        <v>804</v>
+        <v>502</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="1">
-        <v>7577022</v>
+        <v>6056810</v>
       </c>
       <c r="B76" t="s">
         <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D76" s="1">
-        <v>804</v>
+        <v>123</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="1">
-        <v>7460665</v>
+        <v>6066691</v>
       </c>
       <c r="B77" t="s">
         <v>4</v>
       </c>
       <c r="C77" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="D77" s="1">
-        <v>804</v>
+        <v>121</v>
       </c>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="1">
-        <v>6607068</v>
+        <v>6074386</v>
       </c>
       <c r="B78" t="s">
         <v>4</v>
       </c>
       <c r="C78" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D78" s="1">
-        <v>802</v>
+        <v>402</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="1">
-        <v>6954115</v>
+        <v>6084717</v>
       </c>
       <c r="B79" t="s">
         <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D79" s="1">
-        <v>802</v>
+        <v>804</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="1">
-        <v>5382299</v>
+        <v>6101274</v>
       </c>
       <c r="B80" t="s">
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D80" s="1">
-        <v>802</v>
+        <v>301</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="1">
-        <v>7513900</v>
+        <v>6147465</v>
       </c>
       <c r="B81" t="s">
         <v>4</v>
       </c>
       <c r="C81" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D81" s="1">
-        <v>802</v>
+        <v>505</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="1">
-        <v>6139260</v>
+        <v>6163507</v>
       </c>
       <c r="B82" t="s">
         <v>4</v>
       </c>
       <c r="C82" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="D82" s="1">
-        <v>802</v>
+        <v>502</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="1">
-        <v>6982248</v>
+        <v>6163545</v>
       </c>
       <c r="B83" t="s">
         <v>4</v>
       </c>
       <c r="C83" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="D83" s="1">
-        <v>802</v>
+        <v>502</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="1">
-        <v>7560014</v>
+        <v>6163546</v>
       </c>
       <c r="B84" t="s">
         <v>4</v>
       </c>
       <c r="C84" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D84" s="1">
-        <v>114</v>
+        <v>501</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="1">
-        <v>7375146</v>
+        <v>6163577</v>
       </c>
       <c r="B85" t="s">
         <v>4</v>
       </c>
       <c r="C85" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D85" s="1">
-        <v>114</v>
+        <v>502</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="1">
-        <v>6285090</v>
+        <v>6163586</v>
       </c>
       <c r="B86" t="s">
         <v>4</v>
       </c>
       <c r="C86" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D86" s="1">
-        <v>604</v>
+        <v>502</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="1">
-        <v>3055103</v>
+        <v>6176923</v>
       </c>
       <c r="B87" t="s">
         <v>4</v>
       </c>
       <c r="C87" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D87" s="1">
-        <v>604</v>
+        <v>501</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="1">
-        <v>7457647</v>
+        <v>6181545</v>
       </c>
       <c r="B88" t="s">
         <v>4</v>
       </c>
       <c r="C88" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D88" s="1">
-        <v>604</v>
+        <v>805</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="1">
-        <v>6270833</v>
+        <v>6196210</v>
       </c>
       <c r="B89" t="s">
         <v>4</v>
       </c>
       <c r="C89" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D89" s="1">
-        <v>307</v>
+        <v>503</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="1">
-        <v>6410802</v>
+        <v>6196763</v>
       </c>
       <c r="B90" t="s">
         <v>4</v>
       </c>
       <c r="C90" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D90" s="1">
-        <v>307</v>
+        <v>503</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="1">
-        <v>7510353</v>
+        <v>6199900</v>
       </c>
       <c r="B91" t="s">
         <v>4</v>
       </c>
       <c r="C91" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D91" s="1">
-        <v>307</v>
+        <v>505</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="1">
-        <v>7235596</v>
+        <v>620793</v>
       </c>
       <c r="B92" t="s">
         <v>4</v>
       </c>
       <c r="C92" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="D92" s="1">
-        <v>307</v>
+        <v>134</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="1">
-        <v>2878257</v>
+        <v>6224963</v>
       </c>
       <c r="B93" t="s">
         <v>4</v>
       </c>
       <c r="C93" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D93" s="1">
-        <v>307</v>
+        <v>501</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="1">
-        <v>7500702</v>
+        <v>6245269</v>
       </c>
       <c r="B94" t="s">
         <v>4</v>
       </c>
       <c r="C94" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D94" s="1">
-        <v>307</v>
+        <v>505</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="1">
-        <v>6344857</v>
+        <v>6270833</v>
       </c>
       <c r="B95" t="s">
         <v>4</v>
       </c>
       <c r="C95" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D95" s="1">
         <v>307</v>
@@ -1816,27 +1830,27 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="1">
-        <v>5510670</v>
+        <v>6318281</v>
       </c>
       <c r="B96" t="s">
         <v>4</v>
       </c>
       <c r="C96" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D96" s="1">
-        <v>603</v>
+        <v>140</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="1">
-        <v>6221599</v>
+        <v>6344988</v>
       </c>
       <c r="B97" t="s">
         <v>4</v>
       </c>
       <c r="C97" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D97" s="1">
         <v>505</v>
@@ -1844,55 +1858,55 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="1">
-        <v>5538095</v>
+        <v>637697</v>
       </c>
       <c r="B98" t="s">
         <v>4</v>
       </c>
       <c r="C98" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D98" s="1">
-        <v>505</v>
+        <v>805</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="1">
-        <v>5455252</v>
+        <v>640174</v>
       </c>
       <c r="B99" t="s">
         <v>4</v>
       </c>
       <c r="C99" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D99" s="1">
-        <v>505</v>
+        <v>803</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="1">
-        <v>6285788</v>
+        <v>6425620</v>
       </c>
       <c r="B100" t="s">
         <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D100" s="1">
-        <v>505</v>
+        <v>501</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="1">
-        <v>5181870</v>
+        <v>6453079</v>
       </c>
       <c r="B101" t="s">
         <v>4</v>
       </c>
       <c r="C101" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D101" s="1">
         <v>505</v>
@@ -1900,105 +1914,105 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="1">
-        <v>6601032</v>
+        <v>6460651</v>
       </c>
       <c r="B102" t="s">
         <v>4</v>
       </c>
       <c r="C102" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D102" s="1">
-        <v>505</v>
+        <v>123</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="1">
-        <v>7068453</v>
+        <v>6466293</v>
       </c>
       <c r="B103" t="s">
         <v>4</v>
       </c>
       <c r="C103" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D103" s="1">
-        <v>505</v>
+        <v>123</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="1">
-        <v>3497654</v>
+        <v>648205</v>
       </c>
       <c r="B104" t="s">
         <v>4</v>
       </c>
       <c r="C104" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D104" s="1">
-        <v>606</v>
+        <v>503</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="1">
-        <v>5891561</v>
+        <v>653437</v>
       </c>
       <c r="B105" t="s">
         <v>4</v>
       </c>
       <c r="C105" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D105" s="1">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="1">
-        <v>6968628</v>
+        <v>6537165</v>
       </c>
       <c r="B106" t="s">
         <v>4</v>
       </c>
       <c r="C106" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D106" s="1">
-        <v>805</v>
+        <v>301</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="1">
-        <v>5230228</v>
+        <v>6537915</v>
       </c>
       <c r="B107" t="s">
         <v>4</v>
       </c>
       <c r="C107" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D107" s="1">
-        <v>805</v>
+        <v>501</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="1">
-        <v>6569618</v>
+        <v>654102</v>
       </c>
       <c r="B108" t="s">
         <v>4</v>
       </c>
       <c r="C108" t="s">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="D108" s="1">
-        <v>805</v>
+        <v>605</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="1">
-        <v>4741123</v>
+        <v>655806</v>
       </c>
       <c r="B109" t="s">
         <v>4</v>
@@ -2007,46 +2021,46 @@
         <v>25</v>
       </c>
       <c r="D109" s="1">
-        <v>805</v>
+        <v>807</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="1">
-        <v>7525177</v>
+        <v>6559789</v>
       </c>
       <c r="B110" t="s">
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D110" s="1">
-        <v>805</v>
+        <v>307</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="1">
-        <v>6567826</v>
+        <v>6567226</v>
       </c>
       <c r="B111" t="s">
         <v>4</v>
       </c>
       <c r="C111" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D111" s="1">
-        <v>805</v>
+        <v>140</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="1">
-        <v>7075120</v>
+        <v>6567826</v>
       </c>
       <c r="B112" t="s">
         <v>4</v>
       </c>
       <c r="C112" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D112" s="1">
         <v>805</v>
@@ -2054,13 +2068,13 @@
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="1">
-        <v>7359806</v>
+        <v>6569618</v>
       </c>
       <c r="B113" t="s">
         <v>4</v>
       </c>
       <c r="C113" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D113" s="1">
         <v>805</v>
@@ -2068,147 +2082,147 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="1">
-        <v>7032346</v>
+        <v>6571893</v>
       </c>
       <c r="B114" t="s">
         <v>4</v>
       </c>
       <c r="C114" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D114" s="1">
-        <v>805</v>
+        <v>502</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="1">
-        <v>7422485</v>
+        <v>6601032</v>
       </c>
       <c r="B115" t="s">
         <v>4</v>
       </c>
       <c r="C115" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D115" s="1">
-        <v>805</v>
+        <v>505</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="1">
-        <v>6181545</v>
+        <v>6605714</v>
       </c>
       <c r="B116" t="s">
         <v>4</v>
       </c>
       <c r="C116" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D116" s="1">
-        <v>805</v>
+        <v>505</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="1">
-        <v>7060208</v>
+        <v>6610701</v>
       </c>
       <c r="B117" t="s">
         <v>4</v>
       </c>
       <c r="C117" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D117" s="1">
-        <v>805</v>
+        <v>505</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="1">
-        <v>7215889</v>
+        <v>6616035</v>
       </c>
       <c r="B118" t="s">
         <v>4</v>
       </c>
       <c r="C118" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="D118" s="1">
-        <v>803</v>
+        <v>119</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="1">
-        <v>67689098</v>
+        <v>6625774</v>
       </c>
       <c r="B119" t="s">
         <v>4</v>
       </c>
       <c r="C119" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="D119" s="1">
-        <v>803</v>
+        <v>401</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="1">
-        <v>6047324</v>
+        <v>6631276</v>
       </c>
       <c r="B120" t="s">
         <v>4</v>
       </c>
       <c r="C120" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D120" s="1">
-        <v>803</v>
+        <v>807</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="1">
-        <v>7525440</v>
+        <v>6661891</v>
       </c>
       <c r="B121" t="s">
         <v>4</v>
       </c>
       <c r="C121" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D121" s="1">
-        <v>803</v>
+        <v>501</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="1">
-        <v>7228558</v>
+        <v>6667459</v>
       </c>
       <c r="B122" t="s">
         <v>4</v>
       </c>
       <c r="C122" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D122" s="1">
-        <v>803</v>
+        <v>502</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="1">
-        <v>6931087</v>
+        <v>6673211</v>
       </c>
       <c r="B123" t="s">
         <v>4</v>
       </c>
       <c r="C123" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D123" s="1">
-        <v>803</v>
+        <v>403</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="1">
-        <v>4778297</v>
+        <v>6708754</v>
       </c>
       <c r="B124" t="s">
         <v>4</v>
@@ -2217,12 +2231,12 @@
         <v>26</v>
       </c>
       <c r="D124" s="1">
-        <v>803</v>
+        <v>505</v>
       </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="1">
-        <v>600960</v>
+        <v>6711322</v>
       </c>
       <c r="B125" t="s">
         <v>4</v>
@@ -2231,648 +2245,648 @@
         <v>26</v>
       </c>
       <c r="D125" s="1">
-        <v>803</v>
+        <v>505</v>
       </c>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="1">
-        <v>7344978</v>
+        <v>6720063</v>
       </c>
       <c r="B126" t="s">
         <v>4</v>
       </c>
       <c r="C126" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D126" s="1">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="1">
-        <v>6277523</v>
+        <v>6727318</v>
       </c>
       <c r="B127" t="s">
         <v>4</v>
       </c>
       <c r="C127" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="D127" s="1">
-        <v>803</v>
+        <v>114</v>
       </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="1">
-        <v>3428583</v>
+        <v>6761467</v>
       </c>
       <c r="B128" t="s">
         <v>4</v>
       </c>
       <c r="C128" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D128" s="1">
-        <v>803</v>
+        <v>805</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="1">
-        <v>7576713</v>
+        <v>6794062</v>
       </c>
       <c r="B129" t="s">
         <v>4</v>
       </c>
       <c r="C129" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D129" s="1">
-        <v>803</v>
+        <v>123</v>
       </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="1">
-        <v>3426581</v>
+        <v>6833087</v>
       </c>
       <c r="B130" t="s">
         <v>4</v>
       </c>
       <c r="C130" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D130" s="1">
-        <v>804</v>
+        <v>133</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="1">
-        <v>7289995</v>
+        <v>6876007</v>
       </c>
       <c r="B131" t="s">
         <v>4</v>
       </c>
       <c r="C131" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D131" s="1">
-        <v>804</v>
+        <v>405</v>
       </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="1">
-        <v>7259213</v>
+        <v>6878636</v>
       </c>
       <c r="B132" t="s">
         <v>4</v>
       </c>
       <c r="C132" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D132" s="1">
-        <v>603</v>
+        <v>123</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="1">
-        <v>653294</v>
+        <v>6889564</v>
       </c>
       <c r="B133" t="s">
         <v>4</v>
       </c>
       <c r="C133" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D133" s="1">
-        <v>802</v>
+        <v>505</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="1">
-        <v>3391445</v>
+        <v>6908887</v>
       </c>
       <c r="B134" t="s">
         <v>4</v>
       </c>
       <c r="C134" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D134" s="1">
-        <v>801</v>
+        <v>802</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="1">
-        <v>5252010</v>
+        <v>6917389</v>
       </c>
       <c r="B135" t="s">
         <v>4</v>
       </c>
       <c r="C135" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D135" s="1">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="1">
-        <v>7483745</v>
+        <v>6920776</v>
       </c>
       <c r="B136" t="s">
         <v>4</v>
       </c>
       <c r="C136" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D136" s="1">
-        <v>506</v>
+        <v>501</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="1">
-        <v>6797299</v>
+        <v>6924679</v>
       </c>
       <c r="B137" t="s">
         <v>4</v>
       </c>
       <c r="C137" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D137" s="1">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="1">
-        <v>3373822</v>
+        <v>6931087</v>
       </c>
       <c r="B138" t="s">
         <v>4</v>
       </c>
       <c r="C138" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D138" s="1">
-        <v>403</v>
+        <v>803</v>
       </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="1">
-        <v>3450004</v>
+        <v>6938562</v>
       </c>
       <c r="B139" t="s">
         <v>4</v>
       </c>
       <c r="C139" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D139" s="1">
-        <v>403</v>
+        <v>406</v>
       </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="1">
-        <v>6810964</v>
+        <v>6957152</v>
       </c>
       <c r="B140" t="s">
         <v>4</v>
       </c>
       <c r="C140" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D140" s="1">
-        <v>406</v>
+        <v>804</v>
       </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="1">
-        <v>4054442</v>
+        <v>6957211</v>
       </c>
       <c r="B141" t="s">
         <v>4</v>
       </c>
       <c r="C141" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="D141" s="1">
-        <v>406</v>
+        <v>151</v>
       </c>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="1">
-        <v>3492270</v>
+        <v>6966405</v>
       </c>
       <c r="B142" t="s">
         <v>4</v>
       </c>
       <c r="C142" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D142" s="1">
-        <v>406</v>
+        <v>505</v>
       </c>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="1">
-        <v>7040001</v>
+        <v>7003182</v>
       </c>
       <c r="B143" t="s">
         <v>4</v>
       </c>
       <c r="C143" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D143" s="1">
-        <v>407</v>
+        <v>605</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="1">
-        <v>7230030</v>
+        <v>7016158</v>
       </c>
       <c r="B144" t="s">
         <v>4</v>
       </c>
       <c r="C144" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D144" s="1">
-        <v>407</v>
+        <v>505</v>
       </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="1">
-        <v>7202350</v>
+        <v>7017065</v>
       </c>
       <c r="B145" t="s">
         <v>4</v>
       </c>
       <c r="C145" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D145" s="1">
-        <v>308</v>
+        <v>501</v>
       </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="1">
-        <v>7240100</v>
+        <v>7017742</v>
       </c>
       <c r="B146" t="s">
         <v>4</v>
       </c>
       <c r="C146" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="D146" s="1">
-        <v>308</v>
+        <v>504</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="1">
-        <v>5029711</v>
+        <v>7023240</v>
       </c>
       <c r="B147" t="s">
         <v>4</v>
       </c>
       <c r="C147" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D147" s="1">
-        <v>308</v>
+        <v>301</v>
       </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="1">
-        <v>3062209</v>
+        <v>7029361</v>
       </c>
       <c r="B148" t="s">
         <v>4</v>
       </c>
       <c r="C148" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D148" s="1">
-        <v>308</v>
+        <v>406</v>
       </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="1">
-        <v>3427111</v>
+        <v>7055133</v>
       </c>
       <c r="B149" t="s">
         <v>4</v>
       </c>
       <c r="C149" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D149" s="1">
-        <v>308</v>
+        <v>123</v>
       </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="1">
-        <v>6978244</v>
+        <v>7056949</v>
       </c>
       <c r="B150" t="s">
         <v>4</v>
       </c>
       <c r="C150" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D150" s="1">
-        <v>308</v>
+        <v>140</v>
       </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="1">
-        <v>7038664</v>
+        <v>7056950</v>
       </c>
       <c r="B151" t="s">
         <v>4</v>
       </c>
       <c r="C151" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="D151" s="1">
-        <v>308</v>
+        <v>804</v>
       </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="1">
-        <v>6091016</v>
+        <v>7056964</v>
       </c>
       <c r="B152" t="s">
         <v>4</v>
       </c>
       <c r="C152" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D152" s="1">
-        <v>602</v>
+        <v>505</v>
       </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="1">
-        <v>7023240</v>
+        <v>7056973</v>
       </c>
       <c r="B153" t="s">
         <v>4</v>
       </c>
       <c r="C153" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D153" s="1">
-        <v>605</v>
+        <v>807</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="1">
-        <v>3059109</v>
+        <v>7060208</v>
       </c>
       <c r="B154" t="s">
         <v>4</v>
       </c>
       <c r="C154" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="D154" s="1">
-        <v>201</v>
+        <v>805</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="1">
-        <v>7212855</v>
+        <v>7063232</v>
       </c>
       <c r="B155" t="s">
         <v>4</v>
       </c>
       <c r="C155" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="D155" s="1">
-        <v>201</v>
+        <v>133</v>
       </c>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="1">
-        <v>6705285</v>
+        <v>7064880</v>
       </c>
       <c r="B156" t="s">
         <v>4</v>
       </c>
       <c r="C156" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D156" s="1">
-        <v>201</v>
+        <v>807</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="1">
-        <v>7409656</v>
+        <v>7068453</v>
       </c>
       <c r="B157" t="s">
         <v>4</v>
       </c>
       <c r="C157" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D157" s="1">
-        <v>201</v>
+        <v>505</v>
       </c>
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="1">
-        <v>6949619</v>
+        <v>7074279</v>
       </c>
       <c r="B158" t="s">
         <v>4</v>
       </c>
       <c r="C158" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D158" s="1">
-        <v>201</v>
+        <v>803</v>
       </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="1">
-        <v>5872977</v>
+        <v>7075120</v>
       </c>
       <c r="B159" t="s">
         <v>4</v>
       </c>
       <c r="C159" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="D159" s="1">
-        <v>504</v>
+        <v>805</v>
       </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="1">
-        <v>7545927</v>
+        <v>7087645</v>
       </c>
       <c r="B160" t="s">
         <v>4</v>
       </c>
       <c r="C160" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D160" s="1">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="1">
-        <v>5170837</v>
+        <v>7099959</v>
       </c>
       <c r="B161" t="s">
         <v>4</v>
       </c>
       <c r="C161" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="D161" s="1">
-        <v>504</v>
+        <v>802</v>
       </c>
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="1">
-        <v>5172744</v>
+        <v>7100438</v>
       </c>
       <c r="B162" t="s">
         <v>4</v>
       </c>
       <c r="C162" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="D162" s="1">
-        <v>504</v>
+        <v>802</v>
       </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="1">
-        <v>5817316</v>
+        <v>7209634</v>
       </c>
       <c r="B163" t="s">
         <v>4</v>
       </c>
       <c r="C163" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D163" s="1">
-        <v>406</v>
+        <v>502</v>
       </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="1">
-        <v>924017</v>
+        <v>7215889</v>
       </c>
       <c r="B164" t="s">
         <v>4</v>
       </c>
       <c r="C164" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D164" s="1">
-        <v>123</v>
+        <v>803</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="1">
-        <v>7206189</v>
+        <v>7248689</v>
       </c>
       <c r="B165" t="s">
         <v>4</v>
       </c>
       <c r="C165" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D165" s="1">
-        <v>123</v>
+        <v>505</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="1">
-        <v>3064665</v>
+        <v>7251608</v>
       </c>
       <c r="B166" t="s">
         <v>4</v>
       </c>
       <c r="C166" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D166" s="1">
-        <v>123</v>
+        <v>308</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="1">
-        <v>7055133</v>
+        <v>7252628</v>
       </c>
       <c r="B167" t="s">
         <v>4</v>
       </c>
       <c r="C167" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D167" s="1">
-        <v>123</v>
+        <v>505</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="1">
-        <v>7064958</v>
+        <v>7253399</v>
       </c>
       <c r="B168" t="s">
         <v>4</v>
       </c>
       <c r="C168" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D168" s="1">
-        <v>123</v>
+        <v>505</v>
       </c>
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="1">
-        <v>3990488</v>
+        <v>7254560</v>
       </c>
       <c r="B169" t="s">
         <v>4</v>
       </c>
       <c r="C169" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D169" s="1">
-        <v>123</v>
+        <v>151</v>
       </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="1">
-        <v>5075844</v>
+        <v>7257850</v>
       </c>
       <c r="B170" t="s">
         <v>4</v>
       </c>
       <c r="C170" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D170" s="1">
-        <v>123</v>
+        <v>501</v>
       </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" s="1">
-        <v>7346289</v>
+        <v>7263225</v>
       </c>
       <c r="B171" t="s">
         <v>4</v>
       </c>
       <c r="C171" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D171" s="1">
         <v>123</v>
@@ -2880,100 +2894,688 @@
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="1">
-        <v>7031864</v>
+        <v>7278911</v>
       </c>
       <c r="B172" t="s">
         <v>4</v>
       </c>
       <c r="C172" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D172" s="1">
-        <v>123</v>
+        <v>405</v>
       </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" s="1">
-        <v>5420681</v>
+        <v>7288554</v>
       </c>
       <c r="B173" t="s">
         <v>4</v>
       </c>
       <c r="C173" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D173" s="1">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" s="1">
-        <v>6908570</v>
+        <v>7293077</v>
       </c>
       <c r="B174" t="s">
         <v>4</v>
       </c>
       <c r="C174" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="D174" s="1">
-        <v>123</v>
+        <v>502</v>
       </c>
     </row>
     <row r="175" spans="1:4">
       <c r="A175" s="1">
-        <v>7022850</v>
+        <v>7320518</v>
       </c>
       <c r="B175" t="s">
         <v>4</v>
       </c>
       <c r="C175" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D175" s="1">
-        <v>123</v>
+        <v>501</v>
       </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" s="1">
-        <v>6998774</v>
+        <v>7331992</v>
       </c>
       <c r="B176" t="s">
         <v>4</v>
       </c>
       <c r="C176" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D176" s="1">
-        <v>123</v>
+        <v>805</v>
       </c>
     </row>
     <row r="177" spans="1:4">
       <c r="A177" s="1">
-        <v>3392842</v>
+        <v>7347397</v>
       </c>
       <c r="B177" t="s">
         <v>4</v>
       </c>
       <c r="C177" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D177" s="1">
-        <v>123</v>
+        <v>505</v>
       </c>
     </row>
     <row r="178" spans="1:4">
       <c r="A178" s="1">
-        <v>6794062</v>
+        <v>7349585</v>
       </c>
       <c r="B178" t="s">
         <v>4</v>
       </c>
       <c r="C178" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D178" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4">
+      <c r="A179" s="1">
+        <v>7356413</v>
+      </c>
+      <c r="B179" t="s">
+        <v>4</v>
+      </c>
+      <c r="C179" t="s">
+        <v>30</v>
+      </c>
+      <c r="D179" s="1">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4">
+      <c r="A180" s="1">
+        <v>7369107</v>
+      </c>
+      <c r="B180" t="s">
+        <v>4</v>
+      </c>
+      <c r="C180" t="s">
+        <v>16</v>
+      </c>
+      <c r="D180" s="1">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4">
+      <c r="A181" s="1">
+        <v>7372090</v>
+      </c>
+      <c r="B181" t="s">
+        <v>4</v>
+      </c>
+      <c r="C181" t="s">
+        <v>26</v>
+      </c>
+      <c r="D181" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4">
+      <c r="A182" s="1">
+        <v>7373764</v>
+      </c>
+      <c r="B182" t="s">
+        <v>4</v>
+      </c>
+      <c r="C182" t="s">
+        <v>19</v>
+      </c>
+      <c r="D182" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4">
+      <c r="A183" s="1">
+        <v>7375151</v>
+      </c>
+      <c r="B183" t="s">
+        <v>4</v>
+      </c>
+      <c r="C183" t="s">
+        <v>29</v>
+      </c>
+      <c r="D183" s="1">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4">
+      <c r="A184" s="1">
+        <v>7377788</v>
+      </c>
+      <c r="B184" t="s">
+        <v>4</v>
+      </c>
+      <c r="C184" t="s">
+        <v>33</v>
+      </c>
+      <c r="D184" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4">
+      <c r="A185" s="1">
+        <v>7381353</v>
+      </c>
+      <c r="B185" t="s">
+        <v>4</v>
+      </c>
+      <c r="C185" t="s">
+        <v>26</v>
+      </c>
+      <c r="D185" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4">
+      <c r="A186" s="1">
+        <v>7383228</v>
+      </c>
+      <c r="B186" t="s">
+        <v>4</v>
+      </c>
+      <c r="C186" t="s">
+        <v>36</v>
+      </c>
+      <c r="D186" s="1">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4">
+      <c r="A187" s="1">
+        <v>7400761</v>
+      </c>
+      <c r="B187" t="s">
+        <v>4</v>
+      </c>
+      <c r="C187" t="s">
+        <v>33</v>
+      </c>
+      <c r="D187" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4">
+      <c r="A188" s="1">
+        <v>7407064</v>
+      </c>
+      <c r="B188" t="s">
+        <v>4</v>
+      </c>
+      <c r="C188" t="s">
+        <v>25</v>
+      </c>
+      <c r="D188" s="1">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4">
+      <c r="A189" s="1">
+        <v>7417340</v>
+      </c>
+      <c r="B189" t="s">
+        <v>4</v>
+      </c>
+      <c r="C189" t="s">
+        <v>6</v>
+      </c>
+      <c r="D189" s="1">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4">
+      <c r="A190" s="1">
+        <v>7422485</v>
+      </c>
+      <c r="B190" t="s">
+        <v>4</v>
+      </c>
+      <c r="C190" t="s">
+        <v>19</v>
+      </c>
+      <c r="D190" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4">
+      <c r="A191" s="1">
+        <v>7453548</v>
+      </c>
+      <c r="B191" t="s">
+        <v>4</v>
+      </c>
+      <c r="C191" t="s">
+        <v>8</v>
+      </c>
+      <c r="D191" s="1">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4">
+      <c r="A192" s="1">
+        <v>7454188</v>
+      </c>
+      <c r="B192" t="s">
+        <v>4</v>
+      </c>
+      <c r="C192" t="s">
+        <v>37</v>
+      </c>
+      <c r="D192" s="1">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4">
+      <c r="A193" s="1">
+        <v>7456256</v>
+      </c>
+      <c r="B193" t="s">
+        <v>4</v>
+      </c>
+      <c r="C193" t="s">
+        <v>12</v>
+      </c>
+      <c r="D193" s="1">
         <v>123</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4">
+      <c r="A194" s="1">
+        <v>7462357</v>
+      </c>
+      <c r="B194" t="s">
+        <v>4</v>
+      </c>
+      <c r="C194" t="s">
+        <v>26</v>
+      </c>
+      <c r="D194" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4">
+      <c r="A195" s="1">
+        <v>7462588</v>
+      </c>
+      <c r="B195" t="s">
+        <v>4</v>
+      </c>
+      <c r="C195" t="s">
+        <v>38</v>
+      </c>
+      <c r="D195" s="1">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4">
+      <c r="A196" s="1">
+        <v>7473290</v>
+      </c>
+      <c r="B196" t="s">
+        <v>4</v>
+      </c>
+      <c r="C196" t="s">
+        <v>6</v>
+      </c>
+      <c r="D196" s="1">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4">
+      <c r="A197" s="1">
+        <v>7485080</v>
+      </c>
+      <c r="B197" t="s">
+        <v>4</v>
+      </c>
+      <c r="C197" t="s">
+        <v>37</v>
+      </c>
+      <c r="D197" s="1">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4">
+      <c r="A198" s="1">
+        <v>7490788</v>
+      </c>
+      <c r="B198" t="s">
+        <v>4</v>
+      </c>
+      <c r="C198" t="s">
+        <v>26</v>
+      </c>
+      <c r="D198" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4">
+      <c r="A199" s="1">
+        <v>7490792</v>
+      </c>
+      <c r="B199" t="s">
+        <v>4</v>
+      </c>
+      <c r="C199" t="s">
+        <v>26</v>
+      </c>
+      <c r="D199" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4">
+      <c r="A200" s="1">
+        <v>7498321</v>
+      </c>
+      <c r="B200" t="s">
+        <v>4</v>
+      </c>
+      <c r="C200" t="s">
+        <v>16</v>
+      </c>
+      <c r="D200" s="1">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4">
+      <c r="A201" s="1">
+        <v>7498384</v>
+      </c>
+      <c r="B201" t="s">
+        <v>4</v>
+      </c>
+      <c r="C201" t="s">
+        <v>33</v>
+      </c>
+      <c r="D201" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4">
+      <c r="A202" s="1">
+        <v>7499840</v>
+      </c>
+      <c r="B202" t="s">
+        <v>4</v>
+      </c>
+      <c r="C202" t="s">
+        <v>21</v>
+      </c>
+      <c r="D202" s="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4">
+      <c r="A203" s="1">
+        <v>75023048</v>
+      </c>
+      <c r="B203" t="s">
+        <v>4</v>
+      </c>
+      <c r="C203" t="s">
+        <v>6</v>
+      </c>
+      <c r="D203" s="1">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4">
+      <c r="A204" s="1">
+        <v>7506972</v>
+      </c>
+      <c r="B204" t="s">
+        <v>4</v>
+      </c>
+      <c r="C204" t="s">
+        <v>37</v>
+      </c>
+      <c r="D204" s="1">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4">
+      <c r="A205" s="1">
+        <v>7515658</v>
+      </c>
+      <c r="B205" t="s">
+        <v>4</v>
+      </c>
+      <c r="C205" t="s">
+        <v>22</v>
+      </c>
+      <c r="D205" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4">
+      <c r="A206" s="1">
+        <v>7522962</v>
+      </c>
+      <c r="B206" t="s">
+        <v>4</v>
+      </c>
+      <c r="C206" t="s">
+        <v>33</v>
+      </c>
+      <c r="D206" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4">
+      <c r="A207" s="1">
+        <v>7527011</v>
+      </c>
+      <c r="B207" t="s">
+        <v>4</v>
+      </c>
+      <c r="C207" t="s">
+        <v>25</v>
+      </c>
+      <c r="D207" s="1">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4">
+      <c r="A208" s="1">
+        <v>7534497</v>
+      </c>
+      <c r="B208" t="s">
+        <v>4</v>
+      </c>
+      <c r="C208" t="s">
+        <v>20</v>
+      </c>
+      <c r="D208" s="1">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4">
+      <c r="A209" s="1">
+        <v>7541549</v>
+      </c>
+      <c r="B209" t="s">
+        <v>4</v>
+      </c>
+      <c r="C209" t="s">
+        <v>30</v>
+      </c>
+      <c r="D209" s="1">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4">
+      <c r="A210" s="1">
+        <v>7553536</v>
+      </c>
+      <c r="B210" t="s">
+        <v>4</v>
+      </c>
+      <c r="C210" t="s">
+        <v>30</v>
+      </c>
+      <c r="D210" s="1">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4">
+      <c r="A211" s="1">
+        <v>7566549</v>
+      </c>
+      <c r="B211" t="s">
+        <v>4</v>
+      </c>
+      <c r="C211" t="s">
+        <v>14</v>
+      </c>
+      <c r="D211" s="1">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4">
+      <c r="A212" s="1">
+        <v>7576830</v>
+      </c>
+      <c r="B212" t="s">
+        <v>4</v>
+      </c>
+      <c r="C212" t="s">
+        <v>22</v>
+      </c>
+      <c r="D212" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4">
+      <c r="A213" s="1">
+        <v>7578242</v>
+      </c>
+      <c r="B213" t="s">
+        <v>4</v>
+      </c>
+      <c r="C213" t="s">
+        <v>33</v>
+      </c>
+      <c r="D213" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4">
+      <c r="A214" s="1">
+        <v>7579951</v>
+      </c>
+      <c r="B214" t="s">
+        <v>4</v>
+      </c>
+      <c r="C214" t="s">
+        <v>14</v>
+      </c>
+      <c r="D214" s="1">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4">
+      <c r="A215" s="1">
+        <v>7580294</v>
+      </c>
+      <c r="B215" t="s">
+        <v>4</v>
+      </c>
+      <c r="C215" t="s">
+        <v>26</v>
+      </c>
+      <c r="D215" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4">
+      <c r="A216" s="1">
+        <v>7580296</v>
+      </c>
+      <c r="B216" t="s">
+        <v>4</v>
+      </c>
+      <c r="C216" t="s">
+        <v>26</v>
+      </c>
+      <c r="D216" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4">
+      <c r="A217" s="1">
+        <v>7580304</v>
+      </c>
+      <c r="B217" t="s">
+        <v>4</v>
+      </c>
+      <c r="C217" t="s">
+        <v>26</v>
+      </c>
+      <c r="D217" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4">
+      <c r="A218" s="1">
+        <v>912810</v>
+      </c>
+      <c r="B218" t="s">
+        <v>4</v>
+      </c>
+      <c r="C218" t="s">
+        <v>14</v>
+      </c>
+      <c r="D218" s="1">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4">
+      <c r="A219" s="1">
+        <v>922292</v>
+      </c>
+      <c r="B219" t="s">
+        <v>4</v>
+      </c>
+      <c r="C219" t="s">
+        <v>8</v>
+      </c>
+      <c r="D219" s="1">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4">
+      <c r="A220" s="1">
+        <v>929875</v>
+      </c>
+      <c r="B220" t="s">
+        <v>4</v>
+      </c>
+      <c r="C220" t="s">
+        <v>24</v>
+      </c>
+      <c r="D220" s="1">
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização - Mês automático
</commit_message>
<xml_diff>
--- a/Vendas_Do_Dia.xlsx
+++ b/Vendas_Do_Dia.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="24">
   <si>
     <t>Código</t>
   </si>
@@ -28,85 +28,64 @@
     <t>Código_Vendedor</t>
   </si>
   <si>
-    <t>31/03/2026</t>
-  </si>
-  <si>
-    <t>Daniele</t>
-  </si>
-  <si>
-    <t>Cadu</t>
-  </si>
-  <si>
-    <t>Samuel</t>
-  </si>
-  <si>
-    <t>Jose Jose Vicente</t>
-  </si>
-  <si>
-    <t>Jerques</t>
+    <t>06/04/2026</t>
+  </si>
+  <si>
+    <t>Bruno</t>
+  </si>
+  <si>
+    <t>Camilo</t>
+  </si>
+  <si>
+    <t>Guilherme</t>
   </si>
   <si>
     <t>Suene</t>
   </si>
   <si>
+    <t>Sebastião</t>
+  </si>
+  <si>
     <t>Janaína</t>
   </si>
   <si>
+    <t>Aurélio</t>
+  </si>
+  <si>
+    <t>Maycon</t>
+  </si>
+  <si>
+    <t>Ana Luiza</t>
+  </si>
+  <si>
+    <t>Mateus</t>
+  </si>
+  <si>
+    <t>Filipe Assis</t>
+  </si>
+  <si>
+    <t>Larissa</t>
+  </si>
+  <si>
+    <t>Alexandre</t>
+  </si>
+  <si>
     <t>Kenia</t>
   </si>
   <si>
-    <t>Ana Luiza</t>
-  </si>
-  <si>
     <t>Wellinton</t>
   </si>
   <si>
-    <t>Aurélio</t>
-  </si>
-  <si>
     <t>Leandro</t>
   </si>
   <si>
-    <t>Guilherme</t>
-  </si>
-  <si>
-    <t>Maycon</t>
-  </si>
-  <si>
-    <t>Marcão</t>
-  </si>
-  <si>
-    <t>Ian</t>
+    <t>Manoel</t>
   </si>
   <si>
     <t>Álvaro</t>
   </si>
   <si>
-    <t>Victor Pereira</t>
-  </si>
-  <si>
-    <t>Bruno</t>
-  </si>
-  <si>
-    <t>Davidson</t>
-  </si>
-  <si>
-    <t>Luis Felipe</t>
-  </si>
-  <si>
-    <t>Marcos Vinicius</t>
-  </si>
-  <si>
-    <t>Filipe Assis</t>
-  </si>
-  <si>
-    <t>Caio Edson</t>
-  </si>
-  <si>
-    <t>Victor Prazeres</t>
-  </si>
-  <si>
-    <t>Camilo</t>
+    <t>Caíque Mansur</t>
   </si>
 </sst>
 </file>
@@ -465,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D110"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -490,7 +469,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1">
-        <v>2967240</v>
+        <v>3055286</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -499,12 +478,12 @@
         <v>5</v>
       </c>
       <c r="D2" s="1">
-        <v>201</v>
+        <v>602</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1">
-        <v>3059813</v>
+        <v>3058382</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -513,60 +492,60 @@
         <v>6</v>
       </c>
       <c r="D3" s="1">
-        <v>152</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1">
-        <v>3062495</v>
+        <v>3064627</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" s="1">
-        <v>154</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1">
-        <v>3064694</v>
+        <v>3064817</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1">
-        <v>119</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1">
-        <v>3184288</v>
+        <v>3066127</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D6" s="1">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1">
-        <v>3191550</v>
+        <v>3219069</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D7" s="1">
         <v>123</v>
@@ -574,147 +553,147 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1">
-        <v>3390409</v>
+        <v>3262006</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D8" s="1">
-        <v>503</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1">
-        <v>3390412</v>
+        <v>3390409</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1">
-        <v>134</v>
+        <v>503</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1">
-        <v>3390553</v>
+        <v>3422082</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D10" s="1">
-        <v>154</v>
+        <v>803</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1">
-        <v>3391445</v>
+        <v>3562756</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D11" s="1">
-        <v>603</v>
+        <v>803</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1">
-        <v>3422067</v>
+        <v>3667269</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D12" s="1">
-        <v>805</v>
+        <v>406</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1">
-        <v>3422082</v>
+        <v>3798542</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D13" s="1">
-        <v>803</v>
+        <v>602</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1">
-        <v>3451855</v>
+        <v>3858277</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D14" s="1">
-        <v>807</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1">
-        <v>3478318</v>
+        <v>3858281</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D15" s="1">
-        <v>307</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1">
-        <v>3492347</v>
+        <v>4031528</v>
       </c>
       <c r="B16" t="s">
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D16" s="1">
-        <v>406</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1">
-        <v>3545238</v>
+        <v>5062621</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D17" s="1">
-        <v>140</v>
+        <v>603</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="1">
-        <v>3600184</v>
+        <v>5196721</v>
       </c>
       <c r="B18" t="s">
         <v>4</v>
@@ -723,354 +702,354 @@
         <v>14</v>
       </c>
       <c r="D18" s="1">
-        <v>805</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1">
-        <v>3797987</v>
+        <v>5356214</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D19" s="1">
-        <v>301</v>
+        <v>803</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1">
-        <v>4041724</v>
+        <v>5362565</v>
       </c>
       <c r="B20" t="s">
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D20" s="1">
-        <v>151</v>
+        <v>502</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1">
-        <v>4149525</v>
+        <v>5364427</v>
       </c>
       <c r="B21" t="s">
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D21" s="1">
-        <v>151</v>
+        <v>501</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1">
-        <v>4403306</v>
+        <v>5391047</v>
       </c>
       <c r="B22" t="s">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D22" s="1">
-        <v>606</v>
+        <v>501</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1">
-        <v>4632879</v>
+        <v>5393454</v>
       </c>
       <c r="B23" t="s">
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D23" s="1">
-        <v>602</v>
+        <v>504</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="1">
-        <v>4988663</v>
+        <v>5422564</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D24" s="1">
-        <v>804</v>
+        <v>501</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1">
-        <v>5029898</v>
+        <v>5427865</v>
       </c>
       <c r="B25" t="s">
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D25" s="1">
-        <v>151</v>
+        <v>501</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="1">
-        <v>5075854</v>
+        <v>5444091</v>
       </c>
       <c r="B26" t="s">
         <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D26" s="1">
-        <v>151</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="1">
-        <v>5103516</v>
+        <v>5514551</v>
       </c>
       <c r="B27" t="s">
         <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D27" s="1">
-        <v>154</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="1">
-        <v>5171245</v>
+        <v>5603150</v>
       </c>
       <c r="B28" t="s">
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D28" s="1">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="1">
-        <v>5339882</v>
+        <v>5859055</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D29" s="1">
-        <v>503</v>
+        <v>603</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="1">
-        <v>5356214</v>
+        <v>6069644</v>
       </c>
       <c r="B30" t="s">
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D30" s="1">
-        <v>803</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1">
-        <v>5358895</v>
+        <v>6143190</v>
       </c>
       <c r="B31" t="s">
         <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D31" s="1">
-        <v>406</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1">
-        <v>5466252</v>
+        <v>6181497</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
       </c>
       <c r="C32" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D32" s="1">
-        <v>308</v>
+        <v>504</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1">
-        <v>5496333</v>
+        <v>6181545</v>
       </c>
       <c r="B33" t="s">
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D33" s="1">
-        <v>134</v>
+        <v>805</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1">
-        <v>5497058</v>
+        <v>6196210</v>
       </c>
       <c r="B34" t="s">
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D34" s="1">
-        <v>134</v>
+        <v>503</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1">
-        <v>5510670</v>
+        <v>6196763</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D35" s="1">
-        <v>803</v>
+        <v>503</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1">
-        <v>5857773</v>
+        <v>6212641</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="D36" s="1">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="1">
-        <v>5913508</v>
+        <v>6225643</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D37" s="1">
-        <v>301</v>
+        <v>502</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1">
-        <v>5994404</v>
+        <v>6263735</v>
       </c>
       <c r="B38" t="s">
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D38" s="1">
-        <v>807</v>
+        <v>503</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1">
-        <v>6000485</v>
+        <v>6285699</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D39" s="1">
-        <v>301</v>
+        <v>123</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1">
-        <v>6013477</v>
+        <v>6392361</v>
       </c>
       <c r="B40" t="s">
         <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D40" s="1">
-        <v>201</v>
+        <v>502</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1">
-        <v>6020204</v>
+        <v>6395272</v>
       </c>
       <c r="B41" t="s">
         <v>4</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="D41" s="1">
-        <v>804</v>
+        <v>133</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="1">
-        <v>6029141</v>
+        <v>6412929</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
       </c>
       <c r="C42" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="D42" s="1">
-        <v>151</v>
+        <v>401</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1">
-        <v>6029499</v>
+        <v>6462708</v>
       </c>
       <c r="B43" t="s">
         <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D43" s="1">
         <v>807</v>
@@ -1078,49 +1057,49 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="1">
-        <v>6081781</v>
+        <v>6538545</v>
       </c>
       <c r="B44" t="s">
         <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D44" s="1">
-        <v>503</v>
+        <v>123</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="1">
-        <v>6181545</v>
+        <v>655830</v>
       </c>
       <c r="B45" t="s">
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D45" s="1">
-        <v>805</v>
+        <v>405</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="1">
-        <v>6196210</v>
+        <v>6567826</v>
       </c>
       <c r="B46" t="s">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D46" s="1">
-        <v>503</v>
+        <v>805</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1">
-        <v>6196763</v>
+        <v>6584073</v>
       </c>
       <c r="B47" t="s">
         <v>4</v>
@@ -1129,889 +1108,581 @@
         <v>11</v>
       </c>
       <c r="D47" s="1">
-        <v>503</v>
+        <v>803</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="1">
-        <v>6218651</v>
+        <v>6594697</v>
       </c>
       <c r="B48" t="s">
         <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D48" s="1">
-        <v>301</v>
+        <v>151</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="1">
-        <v>6221599</v>
+        <v>6654271</v>
       </c>
       <c r="B49" t="s">
         <v>4</v>
       </c>
       <c r="C49" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D49" s="1">
-        <v>505</v>
+        <v>134</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="1">
-        <v>6261478</v>
+        <v>6676614</v>
       </c>
       <c r="B50" t="s">
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D50" s="1">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="1">
-        <v>6263620</v>
+        <v>6705108</v>
       </c>
       <c r="B51" t="s">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D51" s="1">
-        <v>201</v>
+        <v>133</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="1">
-        <v>628880</v>
+        <v>6712504</v>
       </c>
       <c r="B52" t="s">
         <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D52" s="1">
-        <v>803</v>
+        <v>406</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="1">
-        <v>6384716</v>
+        <v>6741054</v>
       </c>
       <c r="B53" t="s">
         <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D53" s="1">
-        <v>201</v>
+        <v>123</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="1">
-        <v>6411926</v>
+        <v>6751369</v>
       </c>
       <c r="B54" t="s">
         <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="D54" s="1">
-        <v>804</v>
+        <v>133</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="1">
-        <v>652477</v>
+        <v>6870413</v>
       </c>
       <c r="B55" t="s">
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D55" s="1">
-        <v>803</v>
+        <v>123</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="1">
-        <v>652630</v>
+        <v>6908570</v>
       </c>
       <c r="B56" t="s">
         <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D56" s="1">
-        <v>201</v>
+        <v>123</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="1">
-        <v>6574680</v>
+        <v>6910808</v>
       </c>
       <c r="B57" t="s">
         <v>4</v>
       </c>
       <c r="C57" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D57" s="1">
-        <v>605</v>
+        <v>133</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="1">
-        <v>6631276</v>
+        <v>6919069</v>
       </c>
       <c r="B58" t="s">
         <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D58" s="1">
-        <v>807</v>
+        <v>502</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="1">
-        <v>6683400</v>
+        <v>6920023</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="D59" s="1">
-        <v>801</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="1">
-        <v>6702370</v>
+        <v>6931087</v>
       </c>
       <c r="B60" t="s">
         <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D60" s="1">
-        <v>154</v>
+        <v>803</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="1">
-        <v>6712715</v>
+        <v>6935745</v>
       </c>
       <c r="B61" t="s">
         <v>4</v>
       </c>
       <c r="C61" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D61" s="1">
-        <v>801</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="1">
-        <v>6768656</v>
+        <v>6995028</v>
       </c>
       <c r="B62" t="s">
         <v>4</v>
       </c>
       <c r="C62" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D62" s="1">
-        <v>301</v>
+        <v>401</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="1">
-        <v>6810964</v>
+        <v>6995113</v>
       </c>
       <c r="B63" t="s">
         <v>4</v>
       </c>
       <c r="C63" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D63" s="1">
-        <v>406</v>
+        <v>805</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="1">
-        <v>6813794</v>
+        <v>7016889</v>
       </c>
       <c r="B64" t="s">
         <v>4</v>
       </c>
       <c r="C64" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D64" s="1">
-        <v>803</v>
+        <v>406</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="1">
-        <v>6851920</v>
+        <v>7022850</v>
       </c>
       <c r="B65" t="s">
         <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D65" s="1">
-        <v>301</v>
+        <v>123</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="1">
-        <v>6889563</v>
+        <v>7034923</v>
       </c>
       <c r="B66" t="s">
         <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D66" s="1">
-        <v>123</v>
+        <v>307</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="1">
-        <v>6925208</v>
+        <v>7055133</v>
       </c>
       <c r="B67" t="s">
         <v>4</v>
       </c>
       <c r="C67" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="D67" s="1">
-        <v>133</v>
+        <v>123</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="1">
-        <v>6951346</v>
+        <v>7056732</v>
       </c>
       <c r="B68" t="s">
         <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D68" s="1">
-        <v>154</v>
+        <v>503</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="1">
-        <v>6957152</v>
+        <v>7075120</v>
       </c>
       <c r="B69" t="s">
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D69" s="1">
-        <v>804</v>
+        <v>805</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="1">
-        <v>6986688</v>
+        <v>7078465</v>
       </c>
       <c r="B70" t="s">
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="D70" s="1">
-        <v>801</v>
+        <v>133</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="1">
-        <v>7001199</v>
+        <v>7088693</v>
       </c>
       <c r="B71" t="s">
         <v>4</v>
       </c>
       <c r="C71" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D71" s="1">
-        <v>805</v>
+        <v>307</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="1">
-        <v>7009846</v>
+        <v>7094100</v>
       </c>
       <c r="B72" t="s">
         <v>4</v>
       </c>
       <c r="C72" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D72" s="1">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="1">
-        <v>7034923</v>
+        <v>7214877</v>
       </c>
       <c r="B73" t="s">
         <v>4</v>
       </c>
       <c r="C73" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="D73" s="1">
-        <v>605</v>
+        <v>401</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="1">
-        <v>7042192</v>
+        <v>7215889</v>
       </c>
       <c r="B74" t="s">
         <v>4</v>
       </c>
       <c r="C74" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D74" s="1">
-        <v>151</v>
+        <v>803</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="1">
-        <v>7055332</v>
+        <v>7231015</v>
       </c>
       <c r="B75" t="s">
         <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D75" s="1">
-        <v>151</v>
+        <v>134</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="1">
-        <v>7060208</v>
+        <v>7291405</v>
       </c>
       <c r="B76" t="s">
         <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D76" s="1">
-        <v>805</v>
+        <v>501</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="1">
-        <v>7074726</v>
+        <v>7294078</v>
       </c>
       <c r="B77" t="s">
         <v>4</v>
       </c>
       <c r="C77" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D77" s="1">
-        <v>603</v>
+        <v>133</v>
       </c>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="1">
-        <v>7076627</v>
+        <v>7349586</v>
       </c>
       <c r="B78" t="s">
         <v>4</v>
       </c>
       <c r="C78" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D78" s="1">
-        <v>807</v>
+        <v>803</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="1">
-        <v>7076629</v>
+        <v>7359639</v>
       </c>
       <c r="B79" t="s">
         <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D79" s="1">
-        <v>803</v>
+        <v>150</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="1">
-        <v>7083432</v>
+        <v>7408988</v>
       </c>
       <c r="B80" t="s">
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D80" s="1">
-        <v>801</v>
+        <v>602</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="1">
-        <v>7094702</v>
+        <v>7453548</v>
       </c>
       <c r="B81" t="s">
         <v>4</v>
       </c>
       <c r="C81" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D81" s="1">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="1">
-        <v>7210097</v>
+        <v>7466260</v>
       </c>
       <c r="B82" t="s">
         <v>4</v>
       </c>
       <c r="C82" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D82" s="1">
-        <v>308</v>
+        <v>803</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="1">
-        <v>7231015</v>
+        <v>7510871</v>
       </c>
       <c r="B83" t="s">
         <v>4</v>
       </c>
       <c r="C83" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D83" s="1">
-        <v>503</v>
+        <v>307</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="1">
-        <v>7234580</v>
+        <v>7536652</v>
       </c>
       <c r="B84" t="s">
         <v>4</v>
       </c>
       <c r="C84" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="D84" s="1">
-        <v>505</v>
+        <v>123</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="1">
-        <v>7253402</v>
+        <v>7538083</v>
       </c>
       <c r="B85" t="s">
         <v>4</v>
       </c>
       <c r="C85" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D85" s="1">
-        <v>803</v>
+        <v>401</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="1">
-        <v>7254410</v>
+        <v>7560015</v>
       </c>
       <c r="B86" t="s">
         <v>4</v>
       </c>
       <c r="C86" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D86" s="1">
-        <v>805</v>
+        <v>401</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="1">
-        <v>7259213</v>
+        <v>7759800</v>
       </c>
       <c r="B87" t="s">
         <v>4</v>
       </c>
       <c r="C87" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D87" s="1">
-        <v>603</v>
+        <v>401</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="1">
-        <v>7262368</v>
+        <v>925489</v>
       </c>
       <c r="B88" t="s">
         <v>4</v>
       </c>
       <c r="C88" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D88" s="1">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4">
-      <c r="A89" s="1">
-        <v>7268376</v>
-      </c>
-      <c r="B89" t="s">
-        <v>4</v>
-      </c>
-      <c r="C89" t="s">
-        <v>7</v>
-      </c>
-      <c r="D89" s="1">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4">
-      <c r="A90" s="1">
-        <v>7299656</v>
-      </c>
-      <c r="B90" t="s">
-        <v>4</v>
-      </c>
-      <c r="C90" t="s">
-        <v>26</v>
-      </c>
-      <c r="D90" s="1">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4">
-      <c r="A91" s="1">
-        <v>7314858</v>
-      </c>
-      <c r="B91" t="s">
-        <v>4</v>
-      </c>
-      <c r="C91" t="s">
-        <v>26</v>
-      </c>
-      <c r="D91" s="1">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4">
-      <c r="A92" s="1">
-        <v>7320762</v>
-      </c>
-      <c r="B92" t="s">
-        <v>4</v>
-      </c>
-      <c r="C92" t="s">
-        <v>29</v>
-      </c>
-      <c r="D92" s="1">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4">
-      <c r="A93" s="1">
-        <v>7332471</v>
-      </c>
-      <c r="B93" t="s">
-        <v>4</v>
-      </c>
-      <c r="C93" t="s">
-        <v>10</v>
-      </c>
-      <c r="D93" s="1">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4">
-      <c r="A94" s="1">
-        <v>7338910</v>
-      </c>
-      <c r="B94" t="s">
-        <v>4</v>
-      </c>
-      <c r="C94" t="s">
-        <v>8</v>
-      </c>
-      <c r="D94" s="1">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4">
-      <c r="A95" s="1">
-        <v>7346289</v>
-      </c>
-      <c r="B95" t="s">
-        <v>4</v>
-      </c>
-      <c r="C95" t="s">
-        <v>10</v>
-      </c>
-      <c r="D95" s="1">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4">
-      <c r="A96" s="1">
-        <v>7408989</v>
-      </c>
-      <c r="B96" t="s">
-        <v>4</v>
-      </c>
-      <c r="C96" t="s">
-        <v>15</v>
-      </c>
-      <c r="D96" s="1">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4">
-      <c r="A97" s="1">
-        <v>7410012</v>
-      </c>
-      <c r="B97" t="s">
-        <v>4</v>
-      </c>
-      <c r="C97" t="s">
-        <v>22</v>
-      </c>
-      <c r="D97" s="1">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4">
-      <c r="A98" s="1">
-        <v>7417333</v>
-      </c>
-      <c r="B98" t="s">
-        <v>4</v>
-      </c>
-      <c r="C98" t="s">
-        <v>19</v>
-      </c>
-      <c r="D98" s="1">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4">
-      <c r="A99" s="1">
-        <v>7422485</v>
-      </c>
-      <c r="B99" t="s">
-        <v>4</v>
-      </c>
-      <c r="C99" t="s">
-        <v>14</v>
-      </c>
-      <c r="D99" s="1">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4">
-      <c r="A100" s="1">
-        <v>7441529</v>
-      </c>
-      <c r="B100" t="s">
-        <v>4</v>
-      </c>
-      <c r="C100" t="s">
-        <v>20</v>
-      </c>
-      <c r="D100" s="1">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4">
-      <c r="A101" s="1">
-        <v>7460660</v>
-      </c>
-      <c r="B101" t="s">
-        <v>4</v>
-      </c>
-      <c r="C101" t="s">
-        <v>29</v>
-      </c>
-      <c r="D101" s="1">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4">
-      <c r="A102" s="1">
-        <v>7462360</v>
-      </c>
-      <c r="B102" t="s">
-        <v>4</v>
-      </c>
-      <c r="C102" t="s">
-        <v>9</v>
-      </c>
-      <c r="D102" s="1">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4">
-      <c r="A103" s="1">
-        <v>7462843</v>
-      </c>
-      <c r="B103" t="s">
-        <v>4</v>
-      </c>
-      <c r="C103" t="s">
-        <v>15</v>
-      </c>
-      <c r="D103" s="1">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4">
-      <c r="A104" s="1">
-        <v>7466260</v>
-      </c>
-      <c r="B104" t="s">
-        <v>4</v>
-      </c>
-      <c r="C104" t="s">
-        <v>15</v>
-      </c>
-      <c r="D104" s="1">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4">
-      <c r="A105" s="1">
-        <v>7514871</v>
-      </c>
-      <c r="B105" t="s">
-        <v>4</v>
-      </c>
-      <c r="C105" t="s">
-        <v>18</v>
-      </c>
-      <c r="D105" s="1">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4">
-      <c r="A106" s="1">
-        <v>7524581</v>
-      </c>
-      <c r="B106" t="s">
-        <v>4</v>
-      </c>
-      <c r="C106" t="s">
-        <v>16</v>
-      </c>
-      <c r="D106" s="1">
-        <v>807</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4">
-      <c r="A107" s="1">
-        <v>7525440</v>
-      </c>
-      <c r="B107" t="s">
-        <v>4</v>
-      </c>
-      <c r="C107" t="s">
-        <v>15</v>
-      </c>
-      <c r="D107" s="1">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4">
-      <c r="A108" s="1">
-        <v>7536106</v>
-      </c>
-      <c r="B108" t="s">
-        <v>4</v>
-      </c>
-      <c r="C108" t="s">
-        <v>25</v>
-      </c>
-      <c r="D108" s="1">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4">
-      <c r="A109" s="1">
-        <v>7545965</v>
-      </c>
-      <c r="B109" t="s">
-        <v>4</v>
-      </c>
-      <c r="C109" t="s">
-        <v>13</v>
-      </c>
-      <c r="D109" s="1">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4">
-      <c r="A110" s="1">
-        <v>7580296</v>
-      </c>
-      <c r="B110" t="s">
-        <v>4</v>
-      </c>
-      <c r="C110" t="s">
-        <v>25</v>
-      </c>
-      <c r="D110" s="1">
-        <v>505</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizando pastas e pacotes para instalar em outras máquinas com um .exe apenas
</commit_message>
<xml_diff>
--- a/Vendas_Do_Dia.xlsx
+++ b/Vendas_Do_Dia.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="35">
   <si>
     <t>Código</t>
   </si>
@@ -28,64 +28,97 @@
     <t>Código_Vendedor</t>
   </si>
   <si>
-    <t>06/04/2026</t>
+    <t>14/04/2026</t>
+  </si>
+  <si>
+    <t>Camilo</t>
+  </si>
+  <si>
+    <t>Samuel</t>
+  </si>
+  <si>
+    <t>Jose Jose Vicente</t>
+  </si>
+  <si>
+    <t>Lorrane</t>
+  </si>
+  <si>
+    <t>Kenia</t>
+  </si>
+  <si>
+    <t>Suene</t>
+  </si>
+  <si>
+    <t>Victor Prazeres</t>
+  </si>
+  <si>
+    <t>Cadu</t>
+  </si>
+  <si>
+    <t>Wellinton</t>
+  </si>
+  <si>
+    <t>Maycon</t>
+  </si>
+  <si>
+    <t>Marcos Vinicius</t>
+  </si>
+  <si>
+    <t>Ana Luiza</t>
   </si>
   <si>
     <t>Bruno</t>
   </si>
   <si>
-    <t>Camilo</t>
-  </si>
-  <si>
-    <t>Guilherme</t>
-  </si>
-  <si>
-    <t>Suene</t>
+    <t>Davidson</t>
+  </si>
+  <si>
+    <t>Paulo</t>
+  </si>
+  <si>
+    <t>Luis Felipe</t>
+  </si>
+  <si>
+    <t>Alisson</t>
+  </si>
+  <si>
+    <t>Filipe Assis</t>
+  </si>
+  <si>
+    <t>Janaína</t>
+  </si>
+  <si>
+    <t>Leandro</t>
+  </si>
+  <si>
+    <t>Aurélio</t>
+  </si>
+  <si>
+    <t>Alexandre</t>
+  </si>
+  <si>
+    <t>Caíque Mansur</t>
   </si>
   <si>
     <t>Sebastião</t>
   </si>
   <si>
-    <t>Janaína</t>
-  </si>
-  <si>
-    <t>Aurélio</t>
-  </si>
-  <si>
-    <t>Maycon</t>
-  </si>
-  <si>
-    <t>Ana Luiza</t>
-  </si>
-  <si>
-    <t>Mateus</t>
-  </si>
-  <si>
-    <t>Filipe Assis</t>
-  </si>
-  <si>
-    <t>Larissa</t>
-  </si>
-  <si>
-    <t>Alexandre</t>
-  </si>
-  <si>
-    <t>Kenia</t>
-  </si>
-  <si>
-    <t>Wellinton</t>
-  </si>
-  <si>
-    <t>Leandro</t>
-  </si>
-  <si>
-    <t>Manoel</t>
+    <t>Robson</t>
   </si>
   <si>
     <t>Álvaro</t>
   </si>
   <si>
-    <t>Caíque Mansur</t>
+    <t>Ian</t>
+  </si>
+  <si>
+    <t>Michel</t>
+  </si>
+  <si>
+    <t>Monique</t>
+  </si>
+  <si>
+    <t>Victor Pereira</t>
   </si>
 </sst>
 </file>
@@ -444,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D162"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -469,7 +502,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1">
-        <v>3055286</v>
+        <v>3059002</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -478,12 +511,12 @@
         <v>5</v>
       </c>
       <c r="D2" s="1">
-        <v>602</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1">
-        <v>3058382</v>
+        <v>3062495</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -492,180 +525,180 @@
         <v>6</v>
       </c>
       <c r="D3" s="1">
-        <v>133</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1">
-        <v>3064627</v>
+        <v>3064694</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1">
-        <v>133</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1">
-        <v>3064817</v>
+        <v>3179708</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="1">
-        <v>307</v>
+        <v>802</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1">
-        <v>3066127</v>
+        <v>3182900</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D6" s="1">
-        <v>307</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1">
-        <v>3219069</v>
+        <v>3390412</v>
       </c>
       <c r="B7" t="s">
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="1">
-        <v>123</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1">
-        <v>3262006</v>
+        <v>3391323</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1">
-        <v>401</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1">
-        <v>3390409</v>
+        <v>3391445</v>
       </c>
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D9" s="1">
-        <v>503</v>
+        <v>801</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1">
-        <v>3422082</v>
+        <v>3392580</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D10" s="1">
-        <v>803</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1">
-        <v>3562756</v>
+        <v>3450142</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D11" s="1">
-        <v>803</v>
+        <v>805</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1">
-        <v>3667269</v>
+        <v>3472886</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D12" s="1">
-        <v>406</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1">
-        <v>3798542</v>
+        <v>3496853</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D13" s="1">
-        <v>602</v>
+        <v>406</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1">
-        <v>3858277</v>
+        <v>3499292</v>
       </c>
       <c r="B14" t="s">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D14" s="1">
-        <v>133</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1">
-        <v>3858281</v>
+        <v>3520441</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D15" s="1">
-        <v>123</v>
+        <v>603</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1">
-        <v>4031528</v>
+        <v>3633431</v>
       </c>
       <c r="B16" t="s">
         <v>4</v>
@@ -674,298 +707,298 @@
         <v>8</v>
       </c>
       <c r="D16" s="1">
-        <v>123</v>
+        <v>802</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1">
-        <v>5062621</v>
+        <v>3656343</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D17" s="1">
-        <v>603</v>
+        <v>802</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="1">
-        <v>5196721</v>
+        <v>3712213</v>
       </c>
       <c r="B18" t="s">
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="D18" s="1">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1">
-        <v>5356214</v>
+        <v>3770156</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D19" s="1">
-        <v>803</v>
+        <v>603</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1">
-        <v>5362565</v>
+        <v>3990488</v>
       </c>
       <c r="B20" t="s">
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D20" s="1">
-        <v>502</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1">
-        <v>5364427</v>
+        <v>3993265</v>
       </c>
       <c r="B21" t="s">
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D21" s="1">
-        <v>501</v>
+        <v>802</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1">
-        <v>5391047</v>
+        <v>4113134</v>
       </c>
       <c r="B22" t="s">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D22" s="1">
-        <v>501</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="1">
-        <v>5393454</v>
+        <v>4219916</v>
       </c>
       <c r="B23" t="s">
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D23" s="1">
-        <v>504</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="1">
-        <v>5422564</v>
+        <v>4632879</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D24" s="1">
-        <v>501</v>
+        <v>602</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="1">
-        <v>5427865</v>
+        <v>4878897</v>
       </c>
       <c r="B25" t="s">
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D25" s="1">
-        <v>501</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="1">
-        <v>5444091</v>
+        <v>5008509</v>
       </c>
       <c r="B26" t="s">
         <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="D26" s="1">
-        <v>134</v>
+        <v>802</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="1">
-        <v>5514551</v>
+        <v>5110749</v>
       </c>
       <c r="B27" t="s">
         <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D27" s="1">
-        <v>123</v>
+        <v>804</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="1">
-        <v>5603150</v>
+        <v>5139863</v>
       </c>
       <c r="B28" t="s">
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D28" s="1">
-        <v>502</v>
+        <v>804</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="1">
-        <v>5859055</v>
+        <v>5171244</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D29" s="1">
-        <v>603</v>
+        <v>506</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="1">
-        <v>6069644</v>
+        <v>5172140</v>
       </c>
       <c r="B30" t="s">
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D30" s="1">
-        <v>123</v>
+        <v>505</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="1">
-        <v>6143190</v>
+        <v>5174592</v>
       </c>
       <c r="B31" t="s">
         <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D31" s="1">
-        <v>123</v>
+        <v>506</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1">
-        <v>6181497</v>
+        <v>5180414</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
       </c>
       <c r="C32" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D32" s="1">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1">
-        <v>6181545</v>
+        <v>5181870</v>
       </c>
       <c r="B33" t="s">
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D33" s="1">
-        <v>805</v>
+        <v>505</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1">
-        <v>6196210</v>
+        <v>5247297</v>
       </c>
       <c r="B34" t="s">
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D34" s="1">
-        <v>503</v>
+        <v>134</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1">
-        <v>6196763</v>
+        <v>5265114</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D35" s="1">
-        <v>503</v>
+        <v>407</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="1">
-        <v>6212641</v>
+        <v>5312419</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D36" s="1">
-        <v>401</v>
+        <v>805</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="1">
-        <v>6225643</v>
+        <v>5351345</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D37" s="1">
         <v>502</v>
@@ -973,21 +1006,21 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="1">
-        <v>6263735</v>
+        <v>5358895</v>
       </c>
       <c r="B38" t="s">
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D38" s="1">
-        <v>503</v>
+        <v>406</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="1">
-        <v>6285699</v>
+        <v>5382299</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
@@ -996,18 +1029,18 @@
         <v>8</v>
       </c>
       <c r="D39" s="1">
-        <v>123</v>
+        <v>802</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="1">
-        <v>6392361</v>
+        <v>5391043</v>
       </c>
       <c r="B40" t="s">
         <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D40" s="1">
         <v>502</v>
@@ -1015,125 +1048,125 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="1">
-        <v>6395272</v>
+        <v>5430314</v>
       </c>
       <c r="B41" t="s">
         <v>4</v>
       </c>
       <c r="C41" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D41" s="1">
-        <v>133</v>
+        <v>503</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="1">
-        <v>6412929</v>
+        <v>5439556</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
       </c>
       <c r="C42" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D42" s="1">
-        <v>401</v>
+        <v>807</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="1">
-        <v>6462708</v>
+        <v>5496333</v>
       </c>
       <c r="B43" t="s">
         <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D43" s="1">
-        <v>807</v>
+        <v>134</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="1">
-        <v>6538545</v>
+        <v>5510670</v>
       </c>
       <c r="B44" t="s">
         <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D44" s="1">
-        <v>123</v>
+        <v>803</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="1">
-        <v>655830</v>
+        <v>5593493</v>
       </c>
       <c r="B45" t="s">
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D45" s="1">
-        <v>405</v>
+        <v>504</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="1">
-        <v>6567826</v>
+        <v>5634366</v>
       </c>
       <c r="B46" t="s">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D46" s="1">
-        <v>805</v>
+        <v>150</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="1">
-        <v>6584073</v>
+        <v>5682998</v>
       </c>
       <c r="B47" t="s">
         <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D47" s="1">
-        <v>803</v>
+        <v>804</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="1">
-        <v>6594697</v>
+        <v>5684013</v>
       </c>
       <c r="B48" t="s">
         <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D48" s="1">
-        <v>151</v>
+        <v>802</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="1">
-        <v>6654271</v>
+        <v>5859109</v>
       </c>
       <c r="B49" t="s">
         <v>4</v>
       </c>
       <c r="C49" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D49" s="1">
         <v>134</v>
@@ -1141,77 +1174,77 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="1">
-        <v>6676614</v>
+        <v>5980771</v>
       </c>
       <c r="B50" t="s">
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="D50" s="1">
-        <v>501</v>
+        <v>803</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="1">
-        <v>6705108</v>
+        <v>6006486</v>
       </c>
       <c r="B51" t="s">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="D51" s="1">
-        <v>133</v>
+        <v>803</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="1">
-        <v>6712504</v>
+        <v>6041695</v>
       </c>
       <c r="B52" t="s">
         <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="D52" s="1">
-        <v>406</v>
+        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="1">
-        <v>6741054</v>
+        <v>6041735</v>
       </c>
       <c r="B53" t="s">
         <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D53" s="1">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="1">
-        <v>6751369</v>
+        <v>6047324</v>
       </c>
       <c r="B54" t="s">
         <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="D54" s="1">
-        <v>133</v>
+        <v>803</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="1">
-        <v>6870413</v>
+        <v>6052951</v>
       </c>
       <c r="B55" t="s">
         <v>4</v>
@@ -1220,60 +1253,60 @@
         <v>8</v>
       </c>
       <c r="D55" s="1">
-        <v>123</v>
+        <v>802</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="1">
-        <v>6908570</v>
+        <v>6095823</v>
       </c>
       <c r="B56" t="s">
         <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D56" s="1">
-        <v>123</v>
+        <v>404</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="1">
-        <v>6910808</v>
+        <v>6173709</v>
       </c>
       <c r="B57" t="s">
         <v>4</v>
       </c>
       <c r="C57" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D57" s="1">
-        <v>133</v>
+        <v>123</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="1">
-        <v>6919069</v>
+        <v>6191761</v>
       </c>
       <c r="B58" t="s">
         <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D58" s="1">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="1">
-        <v>6920023</v>
+        <v>6195213</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D59" s="1">
         <v>133</v>
@@ -1281,21 +1314,21 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="1">
-        <v>6931087</v>
+        <v>6196846</v>
       </c>
       <c r="B60" t="s">
         <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D60" s="1">
-        <v>803</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="1">
-        <v>6935745</v>
+        <v>6216577</v>
       </c>
       <c r="B61" t="s">
         <v>4</v>
@@ -1304,292 +1337,292 @@
         <v>8</v>
       </c>
       <c r="D61" s="1">
-        <v>123</v>
+        <v>802</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="1">
-        <v>6995028</v>
+        <v>6219354</v>
       </c>
       <c r="B62" t="s">
         <v>4</v>
       </c>
       <c r="C62" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D62" s="1">
-        <v>401</v>
+        <v>801</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="1">
-        <v>6995113</v>
+        <v>6245269</v>
       </c>
       <c r="B63" t="s">
         <v>4</v>
       </c>
       <c r="C63" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D63" s="1">
-        <v>805</v>
+        <v>505</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="1">
-        <v>7016889</v>
+        <v>6266859</v>
       </c>
       <c r="B64" t="s">
         <v>4</v>
       </c>
       <c r="C64" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D64" s="1">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="1">
-        <v>7022850</v>
+        <v>6333708</v>
       </c>
       <c r="B65" t="s">
         <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D65" s="1">
-        <v>123</v>
+        <v>150</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="1">
-        <v>7034923</v>
+        <v>6334222</v>
       </c>
       <c r="B66" t="s">
         <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D66" s="1">
-        <v>307</v>
+        <v>123</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="1">
-        <v>7055133</v>
+        <v>6334416</v>
       </c>
       <c r="B67" t="s">
         <v>4</v>
       </c>
       <c r="C67" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D67" s="1">
-        <v>123</v>
+        <v>804</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="1">
-        <v>7056732</v>
+        <v>6341224</v>
       </c>
       <c r="B68" t="s">
         <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="D68" s="1">
-        <v>503</v>
+        <v>150</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="1">
-        <v>7075120</v>
+        <v>6412929</v>
       </c>
       <c r="B69" t="s">
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D69" s="1">
-        <v>805</v>
+        <v>401</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="1">
-        <v>7078465</v>
+        <v>6453207</v>
       </c>
       <c r="B70" t="s">
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D70" s="1">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="1">
-        <v>7088693</v>
+        <v>6465186</v>
       </c>
       <c r="B71" t="s">
         <v>4</v>
       </c>
       <c r="C71" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D71" s="1">
-        <v>307</v>
+        <v>802</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="1">
-        <v>7094100</v>
+        <v>6471788</v>
       </c>
       <c r="B72" t="s">
         <v>4</v>
       </c>
       <c r="C72" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="D72" s="1">
-        <v>133</v>
+        <v>803</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="1">
-        <v>7214877</v>
+        <v>653294</v>
       </c>
       <c r="B73" t="s">
         <v>4</v>
       </c>
       <c r="C73" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D73" s="1">
-        <v>401</v>
+        <v>802</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="1">
-        <v>7215889</v>
+        <v>6534894</v>
       </c>
       <c r="B74" t="s">
         <v>4</v>
       </c>
       <c r="C74" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D74" s="1">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="1">
-        <v>7231015</v>
+        <v>653526</v>
       </c>
       <c r="B75" t="s">
         <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="D75" s="1">
-        <v>134</v>
+        <v>403</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="1">
-        <v>7291405</v>
+        <v>654038</v>
       </c>
       <c r="B76" t="s">
         <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D76" s="1">
-        <v>501</v>
+        <v>123</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="1">
-        <v>7294078</v>
+        <v>6567826</v>
       </c>
       <c r="B77" t="s">
         <v>4</v>
       </c>
       <c r="C77" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D77" s="1">
-        <v>133</v>
+        <v>805</v>
       </c>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="1">
-        <v>7349586</v>
+        <v>6585333</v>
       </c>
       <c r="B78" t="s">
         <v>4</v>
       </c>
       <c r="C78" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D78" s="1">
-        <v>803</v>
+        <v>603</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="1">
-        <v>7359639</v>
+        <v>6616254</v>
       </c>
       <c r="B79" t="s">
         <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D79" s="1">
-        <v>150</v>
+        <v>505</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="1">
-        <v>7408988</v>
+        <v>6656327</v>
       </c>
       <c r="B80" t="s">
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D80" s="1">
-        <v>602</v>
+        <v>802</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="1">
-        <v>7453548</v>
+        <v>6673609</v>
       </c>
       <c r="B81" t="s">
         <v>4</v>
       </c>
       <c r="C81" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="D81" s="1">
-        <v>602</v>
+        <v>804</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="1">
-        <v>7466260</v>
+        <v>6683400</v>
       </c>
       <c r="B82" t="s">
         <v>4</v>
@@ -1598,91 +1631,1127 @@
         <v>11</v>
       </c>
       <c r="D82" s="1">
-        <v>803</v>
+        <v>801</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="1">
-        <v>7510871</v>
+        <v>6713369</v>
       </c>
       <c r="B83" t="s">
         <v>4</v>
       </c>
       <c r="C83" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D83" s="1">
-        <v>307</v>
+        <v>506</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="1">
-        <v>7536652</v>
+        <v>6746414</v>
       </c>
       <c r="B84" t="s">
         <v>4</v>
       </c>
       <c r="C84" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D84" s="1">
-        <v>123</v>
+        <v>133</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="1">
-        <v>7538083</v>
+        <v>6760710</v>
       </c>
       <c r="B85" t="s">
         <v>4</v>
       </c>
       <c r="C85" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D85" s="1">
-        <v>401</v>
+        <v>133</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="1">
-        <v>7560015</v>
+        <v>6779089</v>
       </c>
       <c r="B86" t="s">
         <v>4</v>
       </c>
       <c r="C86" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="D86" s="1">
-        <v>401</v>
+        <v>151</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="1">
-        <v>7759800</v>
+        <v>6779095</v>
       </c>
       <c r="B87" t="s">
         <v>4</v>
       </c>
       <c r="C87" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D87" s="1">
-        <v>401</v>
+        <v>150</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="1">
-        <v>925489</v>
+        <v>6794061</v>
       </c>
       <c r="B88" t="s">
         <v>4</v>
       </c>
       <c r="C88" t="s">
+        <v>9</v>
+      </c>
+      <c r="D88" s="1">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89" s="1">
+        <v>6813796</v>
+      </c>
+      <c r="B89" t="s">
+        <v>4</v>
+      </c>
+      <c r="C89" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" s="1">
+        <v>6887036</v>
+      </c>
+      <c r="B90" t="s">
+        <v>4</v>
+      </c>
+      <c r="C90" t="s">
+        <v>18</v>
+      </c>
+      <c r="D90" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91" s="1">
+        <v>6889809</v>
+      </c>
+      <c r="B91" t="s">
+        <v>4</v>
+      </c>
+      <c r="C91" t="s">
+        <v>18</v>
+      </c>
+      <c r="D91" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" s="1">
+        <v>6893979</v>
+      </c>
+      <c r="B92" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" t="s">
+        <v>21</v>
+      </c>
+      <c r="D92" s="1">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" s="1">
+        <v>6909778</v>
+      </c>
+      <c r="B93" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" t="s">
+        <v>5</v>
+      </c>
+      <c r="D93" s="1">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" s="1">
+        <v>6920023</v>
+      </c>
+      <c r="B94" t="s">
+        <v>4</v>
+      </c>
+      <c r="C94" t="s">
+        <v>5</v>
+      </c>
+      <c r="D94" s="1">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" s="1">
+        <v>6925208</v>
+      </c>
+      <c r="B95" t="s">
+        <v>4</v>
+      </c>
+      <c r="C95" t="s">
+        <v>5</v>
+      </c>
+      <c r="D95" s="1">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" s="1">
+        <v>6931087</v>
+      </c>
+      <c r="B96" t="s">
+        <v>4</v>
+      </c>
+      <c r="C96" t="s">
+        <v>25</v>
+      </c>
+      <c r="D96" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" s="1">
+        <v>6934291</v>
+      </c>
+      <c r="B97" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97" t="s">
+        <v>10</v>
+      </c>
+      <c r="D97" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
+      <c r="A98" s="1">
+        <v>6945571</v>
+      </c>
+      <c r="B98" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98" t="s">
+        <v>8</v>
+      </c>
+      <c r="D98" s="1">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
+      <c r="A99" s="1">
+        <v>6951346</v>
+      </c>
+      <c r="B99" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99" t="s">
+        <v>6</v>
+      </c>
+      <c r="D99" s="1">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
+      <c r="A100" s="1">
+        <v>7009846</v>
+      </c>
+      <c r="B100" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100" t="s">
+        <v>9</v>
+      </c>
+      <c r="D100" s="1">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
+      <c r="A101" s="1">
+        <v>7040001</v>
+      </c>
+      <c r="B101" t="s">
+        <v>4</v>
+      </c>
+      <c r="C101" t="s">
+        <v>21</v>
+      </c>
+      <c r="D101" s="1">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4">
+      <c r="A102" s="1">
+        <v>7050815</v>
+      </c>
+      <c r="B102" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102" t="s">
+        <v>31</v>
+      </c>
+      <c r="D102" s="1">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
+      <c r="A103" s="1">
+        <v>7052748</v>
+      </c>
+      <c r="B103" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103" t="s">
+        <v>8</v>
+      </c>
+      <c r="D103" s="1">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
+      <c r="A104" s="1">
+        <v>7056945</v>
+      </c>
+      <c r="B104" t="s">
+        <v>4</v>
+      </c>
+      <c r="C104" t="s">
+        <v>10</v>
+      </c>
+      <c r="D104" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4">
+      <c r="A105" s="1">
+        <v>7060208</v>
+      </c>
+      <c r="B105" t="s">
+        <v>4</v>
+      </c>
+      <c r="C105" t="s">
+        <v>13</v>
+      </c>
+      <c r="D105" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4">
+      <c r="A106" s="1">
+        <v>7075120</v>
+      </c>
+      <c r="B106" t="s">
+        <v>4</v>
+      </c>
+      <c r="C106" t="s">
+        <v>13</v>
+      </c>
+      <c r="D106" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4">
+      <c r="A107" s="1">
+        <v>7087047</v>
+      </c>
+      <c r="B107" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" t="s">
+        <v>15</v>
+      </c>
+      <c r="D107" s="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4">
+      <c r="A108" s="1">
+        <v>7088662</v>
+      </c>
+      <c r="B108" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" t="s">
+        <v>8</v>
+      </c>
+      <c r="D108" s="1">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4">
+      <c r="A109" s="1">
+        <v>7097179</v>
+      </c>
+      <c r="B109" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" t="s">
+        <v>32</v>
+      </c>
+      <c r="D109" s="1">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4">
+      <c r="A110" s="1">
+        <v>7103806</v>
+      </c>
+      <c r="B110" t="s">
+        <v>4</v>
+      </c>
+      <c r="C110" t="s">
+        <v>33</v>
+      </c>
+      <c r="D110" s="1">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
+      <c r="A111" s="1">
+        <v>7197164</v>
+      </c>
+      <c r="B111" t="s">
+        <v>4</v>
+      </c>
+      <c r="C111" t="s">
+        <v>13</v>
+      </c>
+      <c r="D111" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
+      <c r="A112" s="1">
+        <v>7209637</v>
+      </c>
+      <c r="B112" t="s">
+        <v>4</v>
+      </c>
+      <c r="C112" t="s">
+        <v>18</v>
+      </c>
+      <c r="D112" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
+      <c r="A113" s="1">
+        <v>7211402</v>
+      </c>
+      <c r="B113" t="s">
+        <v>4</v>
+      </c>
+      <c r="C113" t="s">
+        <v>19</v>
+      </c>
+      <c r="D113" s="1">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
+      <c r="A114" s="1">
+        <v>7215889</v>
+      </c>
+      <c r="B114" t="s">
+        <v>4</v>
+      </c>
+      <c r="C114" t="s">
+        <v>25</v>
+      </c>
+      <c r="D114" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
+      <c r="A115" s="1">
+        <v>7220307</v>
+      </c>
+      <c r="B115" t="s">
+        <v>4</v>
+      </c>
+      <c r="C115" t="s">
+        <v>8</v>
+      </c>
+      <c r="D115" s="1">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
+      <c r="A116" s="1">
+        <v>7230030</v>
+      </c>
+      <c r="B116" t="s">
+        <v>4</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+      <c r="D116" s="1">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
+      <c r="A117" s="1">
+        <v>7235256</v>
+      </c>
+      <c r="B117" t="s">
+        <v>4</v>
+      </c>
+      <c r="C117" t="s">
+        <v>18</v>
+      </c>
+      <c r="D117" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4">
+      <c r="A118" s="1">
+        <v>7254139</v>
+      </c>
+      <c r="B118" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" t="s">
+        <v>27</v>
+      </c>
+      <c r="D118" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
+      <c r="A119" s="1">
+        <v>7254536</v>
+      </c>
+      <c r="B119" t="s">
+        <v>4</v>
+      </c>
+      <c r="C119" t="s">
+        <v>11</v>
+      </c>
+      <c r="D119" s="1">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4">
+      <c r="A120" s="1">
+        <v>7280055</v>
+      </c>
+      <c r="B120" t="s">
+        <v>4</v>
+      </c>
+      <c r="C120" t="s">
+        <v>11</v>
+      </c>
+      <c r="D120" s="1">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
+      <c r="A121" s="1">
+        <v>7281112</v>
+      </c>
+      <c r="B121" t="s">
+        <v>4</v>
+      </c>
+      <c r="C121" t="s">
+        <v>8</v>
+      </c>
+      <c r="D121" s="1">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
+      <c r="A122" s="1">
+        <v>7283541</v>
+      </c>
+      <c r="B122" t="s">
+        <v>4</v>
+      </c>
+      <c r="C122" t="s">
+        <v>20</v>
+      </c>
+      <c r="D122" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
+      <c r="A123" s="1">
+        <v>7285052</v>
+      </c>
+      <c r="B123" t="s">
+        <v>4</v>
+      </c>
+      <c r="C123" t="s">
+        <v>9</v>
+      </c>
+      <c r="D123" s="1">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124" s="1">
+        <v>7289197</v>
+      </c>
+      <c r="B124" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" t="s">
+        <v>25</v>
+      </c>
+      <c r="D124" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4">
+      <c r="A125" s="1">
+        <v>7299656</v>
+      </c>
+      <c r="B125" t="s">
+        <v>4</v>
+      </c>
+      <c r="C125" t="s">
+        <v>15</v>
+      </c>
+      <c r="D125" s="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4">
+      <c r="A126" s="1">
+        <v>7334910</v>
+      </c>
+      <c r="B126" t="s">
+        <v>4</v>
+      </c>
+      <c r="C126" t="s">
+        <v>25</v>
+      </c>
+      <c r="D126" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4">
+      <c r="A127" s="1">
+        <v>7338910</v>
+      </c>
+      <c r="B127" t="s">
+        <v>4</v>
+      </c>
+      <c r="C127" t="s">
+        <v>7</v>
+      </c>
+      <c r="D127" s="1">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" s="1">
+        <v>7348026</v>
+      </c>
+      <c r="B128" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" t="s">
+        <v>10</v>
+      </c>
+      <c r="D128" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
+      <c r="A129" s="1">
+        <v>7371352</v>
+      </c>
+      <c r="B129" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" t="s">
+        <v>10</v>
+      </c>
+      <c r="D129" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4">
+      <c r="A130" s="1">
+        <v>7373088</v>
+      </c>
+      <c r="B130" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" t="s">
+        <v>17</v>
+      </c>
+      <c r="D130" s="1">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" s="1">
+        <v>7408988</v>
+      </c>
+      <c r="B131" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" t="s">
+        <v>17</v>
+      </c>
+      <c r="D131" s="1">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" s="1">
+        <v>7410012</v>
+      </c>
+      <c r="B132" t="s">
+        <v>4</v>
+      </c>
+      <c r="C132" t="s">
+        <v>34</v>
+      </c>
+      <c r="D132" s="1">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" s="1">
+        <v>7416881</v>
+      </c>
+      <c r="B133" t="s">
+        <v>4</v>
+      </c>
+      <c r="C133" t="s">
+        <v>15</v>
+      </c>
+      <c r="D133" s="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" s="1">
+        <v>7421583</v>
+      </c>
+      <c r="B134" t="s">
+        <v>4</v>
+      </c>
+      <c r="C134" t="s">
+        <v>6</v>
+      </c>
+      <c r="D134" s="1">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" s="1">
+        <v>7444212</v>
+      </c>
+      <c r="B135" t="s">
+        <v>4</v>
+      </c>
+      <c r="C135" t="s">
+        <v>25</v>
+      </c>
+      <c r="D135" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" s="1">
+        <v>7459822</v>
+      </c>
+      <c r="B136" t="s">
+        <v>4</v>
+      </c>
+      <c r="C136" t="s">
+        <v>33</v>
+      </c>
+      <c r="D136" s="1">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" s="1">
+        <v>7462355</v>
+      </c>
+      <c r="B137" t="s">
+        <v>4</v>
+      </c>
+      <c r="C137" t="s">
+        <v>13</v>
+      </c>
+      <c r="D137" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" s="1">
+        <v>746243</v>
+      </c>
+      <c r="B138" t="s">
+        <v>4</v>
+      </c>
+      <c r="C138" t="s">
+        <v>25</v>
+      </c>
+      <c r="D138" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" s="1">
+        <v>7467061</v>
+      </c>
+      <c r="B139" t="s">
+        <v>4</v>
+      </c>
+      <c r="C139" t="s">
+        <v>5</v>
+      </c>
+      <c r="D139" s="1">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" s="1">
+        <v>7469739</v>
+      </c>
+      <c r="B140" t="s">
+        <v>4</v>
+      </c>
+      <c r="C140" t="s">
+        <v>19</v>
+      </c>
+      <c r="D140" s="1">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" s="1">
+        <v>748989</v>
+      </c>
+      <c r="B141" t="s">
+        <v>4</v>
+      </c>
+      <c r="C141" t="s">
+        <v>25</v>
+      </c>
+      <c r="D141" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4">
+      <c r="A142" s="1">
+        <v>7490784</v>
+      </c>
+      <c r="B142" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" t="s">
+        <v>20</v>
+      </c>
+      <c r="D142" s="1">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" s="1">
+        <v>7506480</v>
+      </c>
+      <c r="B143" t="s">
+        <v>4</v>
+      </c>
+      <c r="C143" t="s">
+        <v>32</v>
+      </c>
+      <c r="D143" s="1">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4">
+      <c r="A144" s="1">
+        <v>7525177</v>
+      </c>
+      <c r="B144" t="s">
+        <v>4</v>
+      </c>
+      <c r="C144" t="s">
+        <v>13</v>
+      </c>
+      <c r="D144" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4">
+      <c r="A145" s="1">
+        <v>7527424</v>
+      </c>
+      <c r="B145" t="s">
+        <v>4</v>
+      </c>
+      <c r="C145" t="s">
+        <v>25</v>
+      </c>
+      <c r="D145" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4">
+      <c r="A146" s="1">
+        <v>7532647</v>
+      </c>
+      <c r="B146" t="s">
+        <v>4</v>
+      </c>
+      <c r="C146" t="s">
+        <v>16</v>
+      </c>
+      <c r="D146" s="1">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4">
+      <c r="A147" s="1">
+        <v>7536652</v>
+      </c>
+      <c r="B147" t="s">
+        <v>4</v>
+      </c>
+      <c r="C147" t="s">
+        <v>10</v>
+      </c>
+      <c r="D147" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4">
+      <c r="A148" s="1">
+        <v>7539807</v>
+      </c>
+      <c r="B148" t="s">
+        <v>4</v>
+      </c>
+      <c r="C148" t="s">
+        <v>19</v>
+      </c>
+      <c r="D148" s="1">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4">
+      <c r="A149" s="1">
+        <v>7559800</v>
+      </c>
+      <c r="B149" t="s">
+        <v>4</v>
+      </c>
+      <c r="C149" t="s">
+        <v>28</v>
+      </c>
+      <c r="D149" s="1">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4">
+      <c r="A150" s="1">
+        <v>7560015</v>
+      </c>
+      <c r="B150" t="s">
+        <v>4</v>
+      </c>
+      <c r="C150" t="s">
+        <v>28</v>
+      </c>
+      <c r="D150" s="1">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4">
+      <c r="A151" s="1">
+        <v>7562175</v>
+      </c>
+      <c r="B151" t="s">
+        <v>4</v>
+      </c>
+      <c r="C151" t="s">
+        <v>25</v>
+      </c>
+      <c r="D151" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4">
+      <c r="A152" s="1">
+        <v>7562505</v>
+      </c>
+      <c r="B152" t="s">
+        <v>4</v>
+      </c>
+      <c r="C152" t="s">
+        <v>18</v>
+      </c>
+      <c r="D152" s="1">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4">
+      <c r="A153" s="1">
+        <v>7577024</v>
+      </c>
+      <c r="B153" t="s">
+        <v>4</v>
+      </c>
+      <c r="C153" t="s">
+        <v>25</v>
+      </c>
+      <c r="D153" s="1">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4">
+      <c r="A154" s="1">
+        <v>7577648</v>
+      </c>
+      <c r="B154" t="s">
+        <v>4</v>
+      </c>
+      <c r="C154" t="s">
+        <v>5</v>
+      </c>
+      <c r="D154" s="1">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4">
+      <c r="A155" s="1">
+        <v>7580283</v>
+      </c>
+      <c r="B155" t="s">
+        <v>4</v>
+      </c>
+      <c r="C155" t="s">
+        <v>26</v>
+      </c>
+      <c r="D155" s="1">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4">
+      <c r="A156" s="1">
+        <v>7583130</v>
+      </c>
+      <c r="B156" t="s">
+        <v>4</v>
+      </c>
+      <c r="C156" t="s">
+        <v>32</v>
+      </c>
+      <c r="D156" s="1">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4">
+      <c r="A157" s="1">
+        <v>7586827</v>
+      </c>
+      <c r="B157" t="s">
+        <v>4</v>
+      </c>
+      <c r="C157" t="s">
+        <v>10</v>
+      </c>
+      <c r="D157" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4">
+      <c r="A158" s="1">
+        <v>7587310</v>
+      </c>
+      <c r="B158" t="s">
+        <v>4</v>
+      </c>
+      <c r="C158" t="s">
+        <v>32</v>
+      </c>
+      <c r="D158" s="1">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4">
+      <c r="A159" s="1">
+        <v>7587681</v>
+      </c>
+      <c r="B159" t="s">
+        <v>4</v>
+      </c>
+      <c r="C159" t="s">
         <v>23</v>
       </c>
-      <c r="D88" s="1">
-        <v>150</v>
+      <c r="D159" s="1">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4">
+      <c r="A160" s="1">
+        <v>872710</v>
+      </c>
+      <c r="B160" t="s">
+        <v>4</v>
+      </c>
+      <c r="C160" t="s">
+        <v>13</v>
+      </c>
+      <c r="D160" s="1">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4">
+      <c r="A161" s="1">
+        <v>924017</v>
+      </c>
+      <c r="B161" t="s">
+        <v>4</v>
+      </c>
+      <c r="C161" t="s">
+        <v>10</v>
+      </c>
+      <c r="D161" s="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4">
+      <c r="A162" s="1">
+        <v>940081</v>
+      </c>
+      <c r="B162" t="s">
+        <v>4</v>
+      </c>
+      <c r="C162" t="s">
+        <v>20</v>
+      </c>
+      <c r="D162" s="1">
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>